<commit_message>
Update the hour log for week 3.
</commit_message>
<xml_diff>
--- a/docs/2.2_P.CoB_Time_registration_for10.xlsx
+++ b/docs/2.2_P.CoB_Time_registration_for10.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shawn\Dev\ClientOnBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5847AE2-04E2-41A7-A3F4-4685AFCA5883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCB9B4D-75F9-45CB-A5B5-FD508C87065D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="64">
   <si>
     <t>Kickoff</t>
   </si>
@@ -205,6 +205,36 @@
   </si>
   <si>
     <t>Total hours</t>
+  </si>
+  <si>
+    <t>Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Reviewing others' work with feedback</t>
+  </si>
+  <si>
+    <t>Rokas</t>
+  </si>
+  <si>
+    <t>Client email</t>
+  </si>
+  <si>
+    <t>Research editor render tech</t>
+  </si>
+  <si>
+    <t>Database setup</t>
+  </si>
+  <si>
+    <t>Authentication on backend</t>
+  </si>
+  <si>
+    <t>Research GitLab integration</t>
+  </si>
+  <si>
+    <t>Authentication on frontend</t>
   </si>
 </sst>
 </file>
@@ -672,6 +702,12 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -680,12 +716,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -812,7 +842,7 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -898,7 +928,7 @@
                   <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -981,10 +1011,10 @@
                   <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11.5</c:v>
+                  <c:v>16.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1070,7 +1100,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1153,10 +1183,10 @@
                   <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.5</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>11.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1242,7 +1272,7 @@
                   <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>11.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1325,10 +1355,10 @@
                   <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.5</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1362,6 +1392,9 @@
               <c:f>Total!$D$9</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Rokas</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
@@ -1405,13 +1438,13 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>2.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1816,28 +1849,28 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>633.5</c:v>
+                  <c:v>724.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>582</c:v>
+                  <c:v>658.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>582</c:v>
+                  <c:v>581</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>582</c:v>
+                  <c:v>581</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>582</c:v>
+                  <c:v>581</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>582</c:v>
+                  <c:v>581</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>582</c:v>
+                  <c:v>581</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>582</c:v>
+                  <c:v>581</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1896,28 +1929,28 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
+                  <c:v>768</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>672</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>588</c:v>
-                </c:pt>
                 <c:pt idx="2">
-                  <c:v>504</c:v>
+                  <c:v>576</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>420</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>336</c:v>
+                  <c:v>384</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>252</c:v>
+                  <c:v>288</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>168</c:v>
+                  <c:v>192</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>84</c:v>
+                  <c:v>96</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3376,32 +3409,32 @@
         <f>Total!$L$1</f>
         <v>Week 8</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -3551,16 +3584,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -3700,16 +3733,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -3849,16 +3882,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -3998,16 +4031,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -4149,16 +4182,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -4300,16 +4333,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -4447,20 +4480,20 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A66" s="12">
+      <c r="A66" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -4602,16 +4635,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -4753,16 +4786,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -4901,17 +4934,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5175,7 +5208,7 @@
       </c>
       <c r="G2" s="3">
         <f>'Week (3)'!$H$10</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H2" s="3">
         <f>'Week (4)'!$H$10</f>
@@ -5199,7 +5232,7 @@
       </c>
       <c r="M2" s="4">
         <f>SUM(E2:L2)</f>
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5218,7 +5251,7 @@
       </c>
       <c r="G3" s="3">
         <f>'Week (3)'!$H$19</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="H3" s="3">
         <f>'Week (4)'!$H$19</f>
@@ -5242,7 +5275,7 @@
       </c>
       <c r="M3" s="4">
         <f t="shared" ref="M3:M5" si="0">SUM(E3:L3)</f>
-        <v>13.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5261,11 +5294,11 @@
       </c>
       <c r="F4" s="3">
         <f>'Week (2)'!$H$28</f>
-        <v>11.5</v>
+        <v>16.5</v>
       </c>
       <c r="G4" s="3">
         <f>'Week (3)'!$H$28</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H4" s="3">
         <f>'Week (4)'!$H$28</f>
@@ -5289,7 +5322,7 @@
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>17.5</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -5308,7 +5341,7 @@
       </c>
       <c r="G5" s="3">
         <f>'Week (3)'!$H$37</f>
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="H5" s="3">
         <f>'Week (4)'!$H$37</f>
@@ -5332,7 +5365,7 @@
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>10.5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5347,11 +5380,11 @@
       </c>
       <c r="F6" s="3">
         <f>'Week (2)'!$H$46</f>
-        <v>9.5</v>
+        <v>13</v>
       </c>
       <c r="G6" s="3">
         <f>'Week (3)'!$H$46</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="H6" s="3">
         <f>'Week (4)'!$H$46</f>
@@ -5375,7 +5408,7 @@
       </c>
       <c r="M6" s="4">
         <f t="shared" ref="M6" si="1">SUM(E6:L6)</f>
-        <v>15.5</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5394,7 +5427,7 @@
       </c>
       <c r="G7" s="3">
         <f>'Week (3)'!$H$55</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="H7" s="3">
         <f>'Week (4)'!$H$55</f>
@@ -5418,7 +5451,7 @@
       </c>
       <c r="M7" s="4">
         <f t="shared" ref="M7:M11" si="2">SUM(E7:L7)</f>
-        <v>14.5</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5433,11 +5466,11 @@
       </c>
       <c r="F8" s="3">
         <f>'Week (2)'!$H$64</f>
-        <v>4.5</v>
+        <v>8</v>
       </c>
       <c r="G8" s="3">
         <f>'Week (3)'!$H$64</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H8" s="3">
         <f>'Week (4)'!$H$64</f>
@@ -5461,24 +5494,26 @@
       </c>
       <c r="M8" s="4">
         <f t="shared" si="2"/>
-        <v>9.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="30"/>
       <c r="B9" s="31"/>
-      <c r="D9" s="16"/>
+      <c r="D9" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="E9" s="3">
         <f>'Week (1)'!$H$75</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F9" s="3">
         <f>'Week (2)'!$H$73</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G9" s="3">
         <f>'Week (3)'!$H$73</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H9" s="3">
         <f>'Week (4)'!$H$73</f>
@@ -5502,7 +5537,7 @@
       </c>
       <c r="M9" s="4">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5595,15 +5630,15 @@
       </c>
       <c r="E12" s="15">
         <f t="shared" ref="E12:L12" si="3">SUM(E2:E11)</f>
-        <v>38.5</v>
+        <v>43.5</v>
       </c>
       <c r="F12" s="15">
         <f t="shared" si="3"/>
-        <v>51.5</v>
+        <v>66</v>
       </c>
       <c r="G12" s="15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>77.5</v>
       </c>
       <c r="H12" s="15">
         <f t="shared" si="3"/>
@@ -5635,12 +5670,12 @@
       <c r="E13" s="20"/>
       <c r="F13" s="20">
         <f>SUM(E2:F11)</f>
-        <v>90</v>
+        <v>109.5</v>
       </c>
       <c r="G13" s="20"/>
       <c r="H13" s="20">
         <f>SUM(G2:H11)</f>
-        <v>0</v>
+        <v>77.5</v>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="20">
@@ -5661,35 +5696,35 @@
       </c>
       <c r="E14" s="18">
         <f>E15-E12</f>
-        <v>633.5</v>
+        <v>724.5</v>
       </c>
       <c r="F14" s="18">
         <f>E14-F12</f>
-        <v>582</v>
+        <v>658.5</v>
       </c>
       <c r="G14" s="18">
         <f t="shared" ref="G14:L14" si="4">F14-G12</f>
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="H14" s="18">
         <f t="shared" si="4"/>
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="I14" s="18">
         <f t="shared" si="4"/>
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J14" s="18">
         <f t="shared" si="4"/>
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="4"/>
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="L14" s="18">
         <f t="shared" si="4"/>
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5698,42 +5733,42 @@
       </c>
       <c r="B15" s="34">
         <f>COUNTIF(D2:D11, "&gt;''" )*12</f>
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>36</v>
       </c>
       <c r="E15" s="18">
         <f t="shared" ref="E15:K15" si="5">$B$15+F15</f>
-        <v>672</v>
+        <v>768</v>
       </c>
       <c r="F15" s="18">
         <f t="shared" si="5"/>
-        <v>588</v>
+        <v>672</v>
       </c>
       <c r="G15" s="18">
         <f t="shared" si="5"/>
-        <v>504</v>
+        <v>576</v>
       </c>
       <c r="H15" s="18">
         <f t="shared" si="5"/>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="I15" s="18">
         <f t="shared" si="5"/>
-        <v>336</v>
+        <v>384</v>
       </c>
       <c r="J15" s="18">
         <f t="shared" si="5"/>
-        <v>252</v>
+        <v>288</v>
       </c>
       <c r="K15" s="18">
         <f t="shared" si="5"/>
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="L15" s="18">
         <f>$B$15</f>
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -6023,30 +6058,30 @@
         <f>Total!$E$1</f>
         <v>Week 1</v>
       </c>
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
@@ -6209,16 +6244,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B13" s="40" t="str">
+      <c r="B13" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C13" s="41"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="44"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="str">
@@ -6369,16 +6404,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B23" s="40" t="str">
+      <c r="B23" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="42"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="44"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="str">
@@ -6528,16 +6563,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B32" s="40" t="str">
+      <c r="B32" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C32" s="41"/>
-      <c r="D32" s="41"/>
-      <c r="E32" s="41"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="41"/>
-      <c r="H32" s="42"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="43"/>
+      <c r="H32" s="44"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="str">
@@ -6685,16 +6720,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B41" s="40" t="str">
+      <c r="B41" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C41" s="41"/>
-      <c r="D41" s="41"/>
-      <c r="E41" s="41"/>
-      <c r="F41" s="41"/>
-      <c r="G41" s="41"/>
-      <c r="H41" s="42"/>
+      <c r="C41" s="43"/>
+      <c r="D41" s="43"/>
+      <c r="E41" s="43"/>
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+      <c r="H41" s="44"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="str">
@@ -6844,16 +6879,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B50" s="40" t="str">
+      <c r="B50" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C50" s="41"/>
-      <c r="D50" s="41"/>
-      <c r="E50" s="41"/>
-      <c r="F50" s="41"/>
-      <c r="G50" s="41"/>
-      <c r="H50" s="42"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="43"/>
+      <c r="E50" s="43"/>
+      <c r="F50" s="43"/>
+      <c r="G50" s="43"/>
+      <c r="H50" s="44"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="str">
@@ -7003,16 +7038,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B59" s="40" t="str">
+      <c r="B59" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C59" s="41"/>
-      <c r="D59" s="41"/>
-      <c r="E59" s="41"/>
-      <c r="F59" s="41"/>
-      <c r="G59" s="41"/>
-      <c r="H59" s="42"/>
+      <c r="C59" s="43"/>
+      <c r="D59" s="43"/>
+      <c r="E59" s="43"/>
+      <c r="F59" s="43"/>
+      <c r="G59" s="43"/>
+      <c r="H59" s="44"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="str">
@@ -7154,20 +7189,20 @@
       </c>
     </row>
     <row r="68" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A68" s="12">
+      <c r="A68" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B68" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B68" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C68" s="41"/>
-      <c r="D68" s="41"/>
-      <c r="E68" s="41"/>
-      <c r="F68" s="41"/>
-      <c r="G68" s="41"/>
-      <c r="H68" s="42"/>
+      <c r="C68" s="43"/>
+      <c r="D68" s="43"/>
+      <c r="E68" s="43"/>
+      <c r="F68" s="43"/>
+      <c r="G68" s="43"/>
+      <c r="H68" s="44"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="str">
@@ -7205,17 +7240,21 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B70" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B70" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C70" s="10"/>
       <c r="D70" s="10"/>
       <c r="E70" s="10"/>
-      <c r="F70" s="10"/>
+      <c r="F70" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G70" s="10"/>
       <c r="H70" s="6">
         <f>SUM(B70:G70)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
@@ -7277,7 +7316,7 @@
       </c>
       <c r="B75" s="11">
         <f t="shared" ref="B75:G75" si="22">SUM(B70:B74)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C75" s="11">
         <f t="shared" si="22"/>
@@ -7293,7 +7332,7 @@
       </c>
       <c r="F75" s="11">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G75" s="11">
         <f t="shared" si="22"/>
@@ -7301,7 +7340,7 @@
       </c>
       <c r="H75" s="11">
         <f>SUM(B75:G75)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -7309,16 +7348,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B77" s="40" t="str">
+      <c r="B77" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C77" s="41"/>
-      <c r="D77" s="41"/>
-      <c r="E77" s="41"/>
-      <c r="F77" s="41"/>
-      <c r="G77" s="41"/>
-      <c r="H77" s="42"/>
+      <c r="C77" s="43"/>
+      <c r="D77" s="43"/>
+      <c r="E77" s="43"/>
+      <c r="F77" s="43"/>
+      <c r="G77" s="43"/>
+      <c r="H77" s="44"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="str">
@@ -7460,16 +7499,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B86" s="40" t="str">
+      <c r="B86" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C86" s="41"/>
-      <c r="D86" s="41"/>
-      <c r="E86" s="41"/>
-      <c r="F86" s="41"/>
-      <c r="G86" s="41"/>
-      <c r="H86" s="42"/>
+      <c r="C86" s="43"/>
+      <c r="D86" s="43"/>
+      <c r="E86" s="43"/>
+      <c r="F86" s="43"/>
+      <c r="G86" s="43"/>
+      <c r="H86" s="44"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="str">
@@ -7608,17 +7647,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B32:H32"/>
     <mergeCell ref="B86:H86"/>
     <mergeCell ref="B41:H41"/>
     <mergeCell ref="B50:H50"/>
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B68:H68"/>
     <mergeCell ref="B77:H77"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B32:H32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7898,32 +7937,32 @@
         <f>Total!$F$1</f>
         <v>Week 2</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -8081,16 +8120,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -8244,16 +8283,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -8347,29 +8386,39 @@
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="9"/>
-      <c r="B26" s="10"/>
+      <c r="A26" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>55</v>
+      </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
+      <c r="G26" s="10">
+        <v>1.5</v>
+      </c>
       <c r="H26" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="9"/>
+      <c r="A27" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10">
+        <v>3.5</v>
+      </c>
       <c r="H27" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="22" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -8399,11 +8448,11 @@
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>11.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -8411,16 +8460,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -8572,16 +8621,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -8656,16 +8705,20 @@
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="9"/>
+      <c r="A43" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
+      <c r="G43" s="10">
+        <v>3.5</v>
+      </c>
       <c r="H43" s="6">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -8721,11 +8774,11 @@
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>9.5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -8733,16 +8786,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -8896,16 +8949,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -8961,16 +9014,20 @@
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
+      <c r="A60" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
       <c r="D60" s="10"/>
       <c r="E60" s="10"/>
       <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
+      <c r="G60" s="10">
+        <v>3.5</v>
+      </c>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -9039,28 +9096,28 @@
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>4.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A66" s="12">
+      <c r="A66" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -9098,9 +9155,11 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
@@ -9108,7 +9167,7 @@
       <c r="G68" s="10"/>
       <c r="H68" s="6">
         <f>SUM(B68:G68)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -9170,7 +9229,7 @@
       </c>
       <c r="B73" s="11">
         <f t="shared" ref="B73:G73" si="19">SUM(B68:B72)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C73" s="11">
         <f t="shared" si="19"/>
@@ -9194,7 +9253,7 @@
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -9202,16 +9261,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -9353,16 +9412,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -9501,17 +9560,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9786,32 +9845,32 @@
         <f>Total!$G$1</f>
         <v>Week 3</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -9848,42 +9907,56 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G5" s="10"/>
       <c r="H5" s="6">
         <f>SUM(B5:G5)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
+      <c r="A6" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
+      <c r="C6" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="6">
         <f t="shared" ref="H6:H9" si="0">SUM(B6:G6)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="9"/>
+      <c r="A7" s="9" t="s">
+        <v>63</v>
+      </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="D7" s="10">
+        <v>1.5</v>
+      </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
       <c r="H7" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -9919,15 +9992,15 @@
       </c>
       <c r="B10" s="11">
         <f t="shared" ref="B10:G10" si="1">SUM(B5:B9)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E10" s="11">
         <f t="shared" si="1"/>
@@ -9935,7 +10008,7 @@
       </c>
       <c r="F10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
@@ -9943,7 +10016,7 @@
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -9961,16 +10034,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -10007,42 +10080,56 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="F14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G14" s="10"/>
       <c r="H14" s="6">
         <f>SUM(B14:G14)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
+      <c r="A15" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
+      <c r="C15" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="6">
         <f t="shared" ref="H15:H18" si="2">SUM(B15:G15)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
+      <c r="A16" s="9" t="s">
+        <v>61</v>
+      </c>
       <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
+      <c r="C16" s="10">
+        <v>1</v>
+      </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -10078,11 +10165,11 @@
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:G19" si="3">SUM(B14:B18)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="D19" s="11">
         <f t="shared" si="3"/>
@@ -10094,7 +10181,7 @@
       </c>
       <c r="F19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
@@ -10102,7 +10189,7 @@
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10110,16 +10197,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -10156,42 +10243,58 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="F23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G23" s="10"/>
       <c r="H23" s="6">
         <f>SUM(B23:G23)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
+      <c r="A24" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="C24" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="6">
         <f t="shared" ref="H24:H27" si="4">SUM(B24:G24)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="9"/>
+      <c r="A25" s="9" t="s">
+        <v>59</v>
+      </c>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="10">
+        <v>1</v>
+      </c>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -10227,11 +10330,11 @@
       </c>
       <c r="B28" s="11">
         <f t="shared" ref="B28:G28" si="5">SUM(B23:B27)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D28" s="11">
         <f t="shared" si="5"/>
@@ -10239,11 +10342,11 @@
       </c>
       <c r="E28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
@@ -10251,7 +10354,7 @@
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10259,16 +10362,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -10305,42 +10408,56 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
+      <c r="A32" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="F32" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G32" s="10"/>
       <c r="H32" s="6">
         <f>SUM(B32:G32)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="9"/>
+      <c r="A33" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
+      <c r="C33" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
       <c r="H33" s="6">
         <f t="shared" ref="H33:H36" si="6">SUM(B33:G33)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="9"/>
+      <c r="A34" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
+      <c r="E34" s="10">
+        <v>3</v>
+      </c>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
       <c r="H34" s="6">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -10376,11 +10493,11 @@
       </c>
       <c r="B37" s="11">
         <f t="shared" ref="B37:G37" si="7">SUM(B32:B36)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D37" s="11">
         <f t="shared" si="7"/>
@@ -10388,11 +10505,11 @@
       </c>
       <c r="E37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G37" s="11">
         <f t="shared" si="7"/>
@@ -10400,7 +10517,7 @@
       </c>
       <c r="H37" s="11">
         <f>SUM(B37:G37)</f>
-        <v>0</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10408,16 +10525,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -10455,43 +10572,59 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B41" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
+      <c r="F41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G41" s="10"/>
       <c r="H41" s="6">
         <f>SUM(B41:G41)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="9"/>
-      <c r="B42" s="10"/>
+      <c r="A42" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" s="10">
+        <v>1.5</v>
+      </c>
       <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
+      <c r="D42" s="10">
+        <v>1</v>
+      </c>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
       <c r="H42" s="6">
         <f t="shared" ref="H42:H45" si="9">SUM(B42:G42)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="9"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="10"/>
+      <c r="A43" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B43" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="C43" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
       <c r="H43" s="6">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -10527,15 +10660,15 @@
       </c>
       <c r="B46" s="11">
         <f t="shared" ref="B46:G46" si="10">SUM(B41:B45)</f>
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="C46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="11">
         <f t="shared" si="10"/>
@@ -10543,7 +10676,7 @@
       </c>
       <c r="F46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
@@ -10551,7 +10684,7 @@
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10559,16 +10692,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -10606,43 +10739,55 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
+      <c r="F50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G50" s="10"/>
       <c r="H50" s="6">
         <f>SUM(B50:G50)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="9"/>
+      <c r="A51" s="9" t="s">
+        <v>60</v>
+      </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
       <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
+      <c r="E51" s="10">
+        <v>4</v>
+      </c>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
       <c r="H51" s="6">
         <f t="shared" ref="H51:H54" si="12">SUM(B51:G51)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" s="9"/>
+      <c r="A52" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
+      <c r="C52" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D52" s="10"/>
       <c r="E52" s="10"/>
       <c r="F52" s="10"/>
       <c r="G52" s="10"/>
       <c r="H52" s="6">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
@@ -10678,11 +10823,11 @@
       </c>
       <c r="B55" s="11">
         <f t="shared" ref="B55:G55" si="13">SUM(B50:B54)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D55" s="11">
         <f t="shared" si="13"/>
@@ -10690,11 +10835,11 @@
       </c>
       <c r="E55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
@@ -10702,7 +10847,7 @@
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10710,16 +10855,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -10757,30 +10902,40 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
+      <c r="F59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G59" s="10"/>
       <c r="H59" s="6">
         <f>SUM(B59:G59)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
+      <c r="A60" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B60" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="C60" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D60" s="10"/>
       <c r="E60" s="10"/>
       <c r="F60" s="10"/>
       <c r="G60" s="10"/>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -10829,11 +10984,11 @@
       </c>
       <c r="B64" s="11">
         <f t="shared" ref="B64:G64" si="16">SUM(B59:B63)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D64" s="11">
         <f t="shared" si="16"/>
@@ -10845,7 +11000,7 @@
       </c>
       <c r="F64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
@@ -10853,24 +11008,24 @@
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A66" s="12">
+      <c r="A66" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -10908,30 +11063,38 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
+      <c r="F68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G68" s="10"/>
       <c r="H68" s="6">
         <f>SUM(B68:G68)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="9"/>
+      <c r="A69" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B69" s="10"/>
-      <c r="C69" s="10"/>
+      <c r="C69" s="10">
+        <v>2.5</v>
+      </c>
       <c r="D69" s="10"/>
       <c r="E69" s="10"/>
       <c r="F69" s="10"/>
       <c r="G69" s="10"/>
       <c r="H69" s="6">
         <f t="shared" ref="H69:H72" si="18">SUM(B69:G69)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -10980,11 +11143,11 @@
       </c>
       <c r="B73" s="11">
         <f t="shared" ref="B73:G73" si="19">SUM(B68:B72)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D73" s="11">
         <f t="shared" si="19"/>
@@ -10996,7 +11159,7 @@
       </c>
       <c r="F73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
@@ -11004,7 +11167,7 @@
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -11012,16 +11175,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -11163,16 +11326,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -11311,17 +11474,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -11596,32 +11759,32 @@
         <f>Total!$H$1</f>
         <v>Week 4</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -11771,16 +11934,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -11920,16 +12083,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -12069,16 +12232,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -12218,16 +12381,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -12369,16 +12532,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -12520,16 +12683,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -12667,20 +12830,20 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A66" s="12">
+      <c r="A66" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -12822,16 +12985,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -12973,16 +13136,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -13121,17 +13284,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -13406,31 +13569,31 @@
         <f>Total!$I$1</f>
         <v>Week 5</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -13580,16 +13743,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -13729,16 +13892,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -13878,16 +14041,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -14027,16 +14190,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -14178,16 +14341,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -14329,16 +14492,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -14476,20 +14639,20 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A66" s="12">
+      <c r="A66" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -14631,16 +14794,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -14782,16 +14945,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -14930,17 +15093,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -15215,32 +15378,32 @@
         <f>Total!$J$1</f>
         <v>Week 6</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -15390,16 +15553,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -15539,16 +15702,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -15688,16 +15851,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -15837,16 +16000,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -15985,16 +16148,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -16136,16 +16299,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -16283,20 +16446,20 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A66" s="12">
+      <c r="A66" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -16438,16 +16601,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -16589,16 +16752,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -16737,17 +16900,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -17022,32 +17185,32 @@
         <f>Total!$K$1</f>
         <v>Week 7</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -17197,16 +17360,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -17346,16 +17509,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -17495,16 +17658,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -17644,16 +17807,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -17795,16 +17958,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -17946,16 +18109,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -18093,20 +18256,20 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
-      <c r="A66" s="12">
+      <c r="A66" s="12" t="str">
         <f>Total!D9</f>
-        <v>0</v>
-      </c>
-      <c r="B66" s="40" t="str">
+        <v>Rokas</v>
+      </c>
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -18248,16 +18411,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -18399,16 +18562,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -18547,17 +18710,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -18565,26 +18728,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <c6664f9864b54a78bdf9e6230de1c78b xmlns="6c73e52c-07d4-4617-ab67-464747257e8d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </c6664f9864b54a78bdf9e6230de1c78b>
-    <Versiebeheer xmlns="ab37b2fe-4f81-426e-b942-40459dbac68c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100294690D6A57C3C4B8650464765815F1C" ma:contentTypeVersion="15" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="bf1d2ff51e740e451b46e7c13bf9e6da">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="45f6ce90-ba85-4ef2-b43f-c64448cd95eb" xmlns:ns3="c7549584-aa9c-449c-abfe-2ca02f3a7188" xmlns:ns4="6c73e52c-07d4-4617-ab67-464747257e8d" xmlns:ns5="ab37b2fe-4f81-426e-b942-40459dbac68c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8575fd65d7959dd12bd4dc11d36e634e" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="45f6ce90-ba85-4ef2-b43f-c64448cd95eb"/>
@@ -18827,26 +18970,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{844B94A5-2CB8-4D3A-A97F-85854BBCA257}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <c6664f9864b54a78bdf9e6230de1c78b xmlns="6c73e52c-07d4-4617-ab67-464747257e8d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </c6664f9864b54a78bdf9e6230de1c78b>
+    <Versiebeheer xmlns="ab37b2fe-4f81-426e-b942-40459dbac68c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477D1558-F7E0-401F-8472-E1151A96BE17}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c73e52c-07d4-4617-ab67-464747257e8d"/>
-    <ds:schemaRef ds:uri="ab37b2fe-4f81-426e-b942-40459dbac68c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{724CCB8E-5E6A-4B8C-A558-5D9223ADF390}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -18865,4 +19009,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477D1558-F7E0-401F-8472-E1151A96BE17}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c73e52c-07d4-4617-ab67-464747257e8d"/>
+    <ds:schemaRef ds:uri="ab37b2fe-4f81-426e-b942-40459dbac68c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{844B94A5-2CB8-4D3A-A97F-85854BBCA257}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the hour log for the 4th week.
</commit_message>
<xml_diff>
--- a/docs/2.2_P.CoB_Time_registration_for10.xlsx
+++ b/docs/2.2_P.CoB_Time_registration_for10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shawn\Dev\ClientOnBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCB9B4D-75F9-45CB-A5B5-FD508C87065D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4F30A3-079A-4FAA-82BC-B9966AEAF819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="75">
   <si>
     <t>Kickoff</t>
   </si>
@@ -235,6 +235,39 @@
   </si>
   <si>
     <t>Authentication on frontend</t>
+  </si>
+  <si>
+    <t>Session page with editor</t>
+  </si>
+  <si>
+    <t>Reviewing work of others + feedback + help</t>
+  </si>
+  <si>
+    <t>Code reviews</t>
+  </si>
+  <si>
+    <t>Session dashboard</t>
+  </si>
+  <si>
+    <t>API request for creating sessions</t>
+  </si>
+  <si>
+    <t>CI workflows</t>
+  </si>
+  <si>
+    <t>Research for websockets</t>
+  </si>
+  <si>
+    <t>User list</t>
+  </si>
+  <si>
+    <t>Frontend on registration page</t>
+  </si>
+  <si>
+    <t>API request for creating a user</t>
+  </si>
+  <si>
+    <t>API request for modifying a user</t>
   </si>
 </sst>
 </file>
@@ -842,10 +875,10 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -928,10 +961,10 @@
                   <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.5</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1014,10 +1047,10 @@
                   <c:v>16.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>11.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1103,7 +1136,7 @@
                   <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1186,10 +1219,10 @@
                   <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>11.5</c:v>
+                  <c:v>12.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1272,10 +1305,10 @@
                   <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>12.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>11.5</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1361,7 +1394,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1447,7 +1480,7 @@
                   <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1855,22 +1888,22 @@
                   <c:v>658.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>581</c:v>
+                  <c:v>572.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>581</c:v>
+                  <c:v>501.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>581</c:v>
+                  <c:v>501.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>581</c:v>
+                  <c:v>501.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>581</c:v>
+                  <c:v>501.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>581</c:v>
+                  <c:v>501.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5208,11 +5241,11 @@
       </c>
       <c r="G2" s="3">
         <f>'Week (3)'!$H$10</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H2" s="3">
         <f>'Week (4)'!$H$10</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I2" s="3">
         <f>'Week (5)'!$H$10</f>
@@ -5232,7 +5265,7 @@
       </c>
       <c r="M2" s="4">
         <f>SUM(E2:L2)</f>
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5251,11 +5284,11 @@
       </c>
       <c r="G3" s="3">
         <f>'Week (3)'!$H$19</f>
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="H3" s="3">
         <f>'Week (4)'!$H$19</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I3" s="3">
         <f>'Week (5)'!$H$19</f>
@@ -5275,7 +5308,7 @@
       </c>
       <c r="M3" s="4">
         <f t="shared" ref="M3:M5" si="0">SUM(E3:L3)</f>
-        <v>22</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5298,11 +5331,11 @@
       </c>
       <c r="G4" s="3">
         <f>'Week (3)'!$H$28</f>
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="H4" s="3">
         <f>'Week (4)'!$H$28</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I4" s="3">
         <f>'Week (5)'!$H$28</f>
@@ -5322,7 +5355,7 @@
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>32.5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -5345,7 +5378,7 @@
       </c>
       <c r="H5" s="3">
         <f>'Week (4)'!$H$37</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I5" s="3">
         <f>'Week (5)'!$H$37</f>
@@ -5365,7 +5398,7 @@
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5384,11 +5417,11 @@
       </c>
       <c r="G6" s="3">
         <f>'Week (3)'!$H$46</f>
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="H6" s="3">
         <f>'Week (4)'!$H$46</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I6" s="3">
         <f>'Week (5)'!$H$46</f>
@@ -5408,7 +5441,7 @@
       </c>
       <c r="M6" s="4">
         <f t="shared" ref="M6" si="1">SUM(E6:L6)</f>
-        <v>30.5</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5427,11 +5460,11 @@
       </c>
       <c r="G7" s="3">
         <f>'Week (3)'!$H$55</f>
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="H7" s="3">
         <f>'Week (4)'!$H$55</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="I7" s="3">
         <f>'Week (5)'!$H$55</f>
@@ -5451,7 +5484,7 @@
       </c>
       <c r="M7" s="4">
         <f t="shared" ref="M7:M11" si="2">SUM(E7:L7)</f>
-        <v>26</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5474,7 +5507,7 @@
       </c>
       <c r="H8" s="3">
         <f>'Week (4)'!$H$64</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I8" s="3">
         <f>'Week (5)'!$H$64</f>
@@ -5494,7 +5527,7 @@
       </c>
       <c r="M8" s="4">
         <f t="shared" si="2"/>
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5517,7 +5550,7 @@
       </c>
       <c r="H9" s="3">
         <f>'Week (4)'!$H$73</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I9" s="3">
         <f>'Week (5)'!$H$73</f>
@@ -5537,7 +5570,7 @@
       </c>
       <c r="M9" s="4">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5638,11 +5671,11 @@
       </c>
       <c r="G12" s="15">
         <f t="shared" si="3"/>
-        <v>77.5</v>
+        <v>86</v>
       </c>
       <c r="H12" s="15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="I12" s="15">
         <f t="shared" si="3"/>
@@ -5675,7 +5708,7 @@
       <c r="G13" s="20"/>
       <c r="H13" s="20">
         <f>SUM(G2:H11)</f>
-        <v>77.5</v>
+        <v>157</v>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="20">
@@ -5704,27 +5737,27 @@
       </c>
       <c r="G14" s="18">
         <f t="shared" ref="G14:L14" si="4">F14-G12</f>
-        <v>581</v>
+        <v>572.5</v>
       </c>
       <c r="H14" s="18">
         <f t="shared" si="4"/>
-        <v>581</v>
+        <v>501.5</v>
       </c>
       <c r="I14" s="18">
         <f t="shared" si="4"/>
-        <v>581</v>
+        <v>501.5</v>
       </c>
       <c r="J14" s="18">
         <f t="shared" si="4"/>
-        <v>581</v>
+        <v>501.5</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="4"/>
-        <v>581</v>
+        <v>501.5</v>
       </c>
       <c r="L14" s="18">
         <f t="shared" si="4"/>
-        <v>581</v>
+        <v>501.5</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9953,10 +9986,12 @@
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+      <c r="G7" s="10">
+        <v>3</v>
+      </c>
       <c r="H7" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -10012,11 +10047,11 @@
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -10133,16 +10168,20 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="9"/>
+      <c r="A17" s="9" t="s">
+        <v>73</v>
+      </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10">
+        <v>2</v>
+      </c>
       <c r="H17" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -10185,11 +10224,11 @@
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10291,10 +10330,12 @@
         <v>1</v>
       </c>
       <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
+      <c r="G25" s="10">
+        <v>1.5</v>
+      </c>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -10350,11 +10391,11 @@
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>10</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10628,16 +10669,20 @@
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="9"/>
+      <c r="A44" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
       <c r="D44" s="10"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
+      <c r="G44" s="10">
+        <v>1</v>
+      </c>
       <c r="H44" s="6">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -10680,11 +10725,11 @@
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -10791,16 +10836,20 @@
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" s="9"/>
+      <c r="A53" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
       <c r="D53" s="10"/>
       <c r="E53" s="10"/>
       <c r="F53" s="10"/>
-      <c r="G53" s="10"/>
+      <c r="G53" s="10">
+        <v>1</v>
+      </c>
       <c r="H53" s="6">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
@@ -10843,11 +10892,11 @@
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -11821,29 +11870,39 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G5" s="10"/>
       <c r="H5" s="6">
         <f>SUM(B5:G5)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
+      <c r="A6" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="E6" s="10">
+        <v>2</v>
+      </c>
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="6">
         <f t="shared" ref="H6:H9" si="0">SUM(B6:G6)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -11892,7 +11951,7 @@
       </c>
       <c r="B10" s="11">
         <f t="shared" ref="B10:G10" si="1">SUM(B5:B9)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C10" s="11">
         <f t="shared" si="1"/>
@@ -11904,11 +11963,11 @@
       </c>
       <c r="E10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
@@ -11916,7 +11975,7 @@
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -11980,29 +12039,39 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="F14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G14" s="10"/>
       <c r="H14" s="6">
         <f>SUM(B14:G14)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
+      <c r="A15" s="9" t="s">
+        <v>74</v>
+      </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
+      <c r="E15" s="10">
+        <v>2.5</v>
+      </c>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="6">
         <f t="shared" ref="H15:H18" si="2">SUM(B15:G15)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
@@ -12051,7 +12120,7 @@
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:G19" si="3">SUM(B14:B18)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="3"/>
@@ -12063,11 +12132,11 @@
       </c>
       <c r="E19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
@@ -12075,7 +12144,7 @@
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -12129,42 +12198,56 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="F23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G23" s="10"/>
       <c r="H23" s="6">
         <f>SUM(B23:G23)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="9"/>
+      <c r="A24" s="9" t="s">
+        <v>64</v>
+      </c>
       <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
+      <c r="C24" s="10">
+        <v>4</v>
+      </c>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="6">
         <f t="shared" ref="H24:H27" si="4">SUM(B24:G24)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="9"/>
+      <c r="A25" s="9" t="s">
+        <v>65</v>
+      </c>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="10">
+        <v>1</v>
+      </c>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -12200,11 +12283,11 @@
       </c>
       <c r="B28" s="11">
         <f t="shared" ref="B28:G28" si="5">SUM(B23:B27)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D28" s="11">
         <f t="shared" si="5"/>
@@ -12212,11 +12295,11 @@
       </c>
       <c r="E28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
@@ -12224,7 +12307,7 @@
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -12278,29 +12361,39 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
+      <c r="A32" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="F32" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G32" s="10"/>
       <c r="H32" s="6">
         <f>SUM(B32:G32)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="9"/>
+      <c r="A33" s="9" t="s">
+        <v>69</v>
+      </c>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
+      <c r="E33" s="10">
+        <v>3</v>
+      </c>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
       <c r="H33" s="6">
         <f t="shared" ref="H33:H36" si="6">SUM(B33:G33)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -12349,7 +12442,7 @@
       </c>
       <c r="B37" s="11">
         <f t="shared" ref="B37:G37" si="7">SUM(B32:B36)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C37" s="11">
         <f t="shared" si="7"/>
@@ -12361,11 +12454,11 @@
       </c>
       <c r="E37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G37" s="11">
         <f t="shared" si="7"/>
@@ -12373,7 +12466,7 @@
       </c>
       <c r="H37" s="11">
         <f>SUM(B37:G37)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -12428,30 +12521,40 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B41" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
+      <c r="F41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G41" s="10"/>
       <c r="H41" s="6">
         <f>SUM(B41:G41)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="9"/>
-      <c r="B42" s="10"/>
+      <c r="A42" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" s="10">
+        <v>3</v>
+      </c>
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
+      <c r="E42" s="10">
+        <v>3</v>
+      </c>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
       <c r="H42" s="6">
         <f t="shared" ref="H42:H45" si="9">SUM(B42:G42)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -12500,7 +12603,7 @@
       </c>
       <c r="B46" s="11">
         <f t="shared" ref="B46:G46" si="10">SUM(B41:B45)</f>
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="C46" s="11">
         <f t="shared" si="10"/>
@@ -12512,11 +12615,11 @@
       </c>
       <c r="E46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
@@ -12524,7 +12627,7 @@
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -12579,43 +12682,55 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
+      <c r="F50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G50" s="10"/>
       <c r="H50" s="6">
         <f>SUM(B50:G50)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="9"/>
+      <c r="A51" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
+      <c r="D51" s="10">
+        <v>3</v>
+      </c>
       <c r="E51" s="10"/>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
       <c r="H51" s="6">
         <f t="shared" ref="H51:H54" si="12">SUM(B51:G51)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" s="9"/>
+      <c r="A52" s="9" t="s">
+        <v>71</v>
+      </c>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
+      <c r="E52" s="10">
+        <v>3.5</v>
+      </c>
       <c r="F52" s="10"/>
       <c r="G52" s="10"/>
       <c r="H52" s="6">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
@@ -12651,7 +12766,7 @@
       </c>
       <c r="B55" s="11">
         <f t="shared" ref="B55:G55" si="13">SUM(B50:B54)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C55" s="11">
         <f t="shared" si="13"/>
@@ -12659,15 +12774,15 @@
       </c>
       <c r="D55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="F55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
@@ -12675,7 +12790,7 @@
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -12730,30 +12845,38 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
+      <c r="F59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G59" s="10"/>
       <c r="H59" s="6">
         <f>SUM(B59:G59)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
+      <c r="A60" s="9" t="s">
+        <v>67</v>
+      </c>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
       <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
+      <c r="E60" s="10">
+        <v>4</v>
+      </c>
       <c r="F60" s="10"/>
       <c r="G60" s="10"/>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -12802,7 +12925,7 @@
       </c>
       <c r="B64" s="11">
         <f t="shared" ref="B64:G64" si="16">SUM(B59:B63)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C64" s="11">
         <f t="shared" si="16"/>
@@ -12814,11 +12937,11 @@
       </c>
       <c r="E64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
@@ -12826,7 +12949,7 @@
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -12881,22 +13004,30 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
+      <c r="F68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G68" s="10"/>
       <c r="H68" s="6">
         <f>SUM(B68:G68)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="9"/>
-      <c r="B69" s="10"/>
+      <c r="A69" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B69" s="10">
+        <v>2</v>
+      </c>
       <c r="C69" s="10"/>
       <c r="D69" s="10"/>
       <c r="E69" s="10"/>
@@ -12904,7 +13035,7 @@
       <c r="G69" s="10"/>
       <c r="H69" s="6">
         <f t="shared" ref="H69:H72" si="18">SUM(B69:G69)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -12953,7 +13084,7 @@
       </c>
       <c r="B73" s="11">
         <f t="shared" ref="B73:G73" si="19">SUM(B68:B72)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="C73" s="11">
         <f t="shared" si="19"/>
@@ -12969,7 +13100,7 @@
       </c>
       <c r="F73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
@@ -12977,7 +13108,7 @@
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update the hour log for the 5th week.
</commit_message>
<xml_diff>
--- a/docs/2.2_P.CoB_Time_registration_for10.xlsx
+++ b/docs/2.2_P.CoB_Time_registration_for10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shawn\Dev\ClientOnBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC4F30A3-079A-4FAA-82BC-B9966AEAF819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AE327A-F333-4DA9-8345-4621810C313F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructie" sheetId="19" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="85">
   <si>
     <t>Kickoff</t>
   </si>
@@ -268,6 +268,36 @@
   </si>
   <si>
     <t>API request for modifying a user</t>
+  </si>
+  <si>
+    <t>Reviewing merge requests</t>
+  </si>
+  <si>
+    <t>Adding nodes in editor</t>
+  </si>
+  <si>
+    <t>API request for creating actions</t>
+  </si>
+  <si>
+    <t>API request for getting past actions</t>
+  </si>
+  <si>
+    <t>API request for obtaining a single user</t>
+  </si>
+  <si>
+    <t>Documenting sprint retrospective</t>
+  </si>
+  <si>
+    <t>Setting up web sockets</t>
+  </si>
+  <si>
+    <t>Appointing and demoting leaders</t>
+  </si>
+  <si>
+    <t>Export to GitLab</t>
+  </si>
+  <si>
+    <t>API request for adding users to a session</t>
   </si>
 </sst>
 </file>
@@ -881,7 +911,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -964,10 +994,10 @@
                   <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.5</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1050,10 +1080,10 @@
                   <c:v>11.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1139,7 +1169,7 @@
                   <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1225,7 +1255,7 @@
                   <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1311,7 +1341,7 @@
                   <c:v>11.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1397,7 +1427,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1483,7 +1513,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1891,19 +1921,19 @@
                   <c:v>572.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>501.5</c:v>
+                  <c:v>499.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>501.5</c:v>
+                  <c:v>435</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>501.5</c:v>
+                  <c:v>435</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>501.5</c:v>
+                  <c:v>435</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>501.5</c:v>
+                  <c:v>435</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5249,7 +5279,7 @@
       </c>
       <c r="I2" s="3">
         <f>'Week (5)'!$H$10</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="J2" s="3">
         <f>'Week (6)'!$H$10</f>
@@ -5265,7 +5295,7 @@
       </c>
       <c r="M2" s="4">
         <f>SUM(E2:L2)</f>
-        <v>28</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5288,11 +5318,11 @@
       </c>
       <c r="H3" s="3">
         <f>'Week (4)'!$H$19</f>
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="I3" s="3">
         <f>'Week (5)'!$H$19</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="J3" s="3">
         <f>'Week (6)'!$H$19</f>
@@ -5308,7 +5338,7 @@
       </c>
       <c r="M3" s="4">
         <f t="shared" ref="M3:M5" si="0">SUM(E3:L3)</f>
-        <v>31.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5335,11 +5365,11 @@
       </c>
       <c r="H4" s="3">
         <f>'Week (4)'!$H$28</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I4" s="3">
         <f>'Week (5)'!$H$28</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J4" s="3">
         <f>'Week (6)'!$H$28</f>
@@ -5355,7 +5385,7 @@
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -5382,7 +5412,7 @@
       </c>
       <c r="I5" s="3">
         <f>'Week (5)'!$H$37</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J5" s="3">
         <f>'Week (6)'!$H$37</f>
@@ -5398,7 +5428,7 @@
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5425,7 +5455,7 @@
       </c>
       <c r="I6" s="3">
         <f>'Week (5)'!$H$46</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="J6" s="3">
         <f>'Week (6)'!$H$46</f>
@@ -5441,7 +5471,7 @@
       </c>
       <c r="M6" s="4">
         <f t="shared" ref="M6" si="1">SUM(E6:L6)</f>
-        <v>42.5</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5468,7 +5498,7 @@
       </c>
       <c r="I7" s="3">
         <f>'Week (5)'!$H$55</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J7" s="3">
         <f>'Week (6)'!$H$55</f>
@@ -5484,7 +5514,7 @@
       </c>
       <c r="M7" s="4">
         <f t="shared" ref="M7:M11" si="2">SUM(E7:L7)</f>
-        <v>38.5</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5511,7 +5541,7 @@
       </c>
       <c r="I8" s="3">
         <f>'Week (5)'!$H$64</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J8" s="3">
         <f>'Week (6)'!$H$64</f>
@@ -5527,7 +5557,7 @@
       </c>
       <c r="M8" s="4">
         <f t="shared" si="2"/>
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5554,7 +5584,7 @@
       </c>
       <c r="I9" s="3">
         <f>'Week (5)'!$H$73</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J9" s="3">
         <f>'Week (6)'!$H$73</f>
@@ -5570,7 +5600,7 @@
       </c>
       <c r="M9" s="4">
         <f t="shared" si="2"/>
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5675,11 +5705,11 @@
       </c>
       <c r="H12" s="15">
         <f t="shared" si="3"/>
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I12" s="15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>64.5</v>
       </c>
       <c r="J12" s="15">
         <f t="shared" si="3"/>
@@ -5708,12 +5738,12 @@
       <c r="G13" s="20"/>
       <c r="H13" s="20">
         <f>SUM(G2:H11)</f>
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="I13" s="20"/>
       <c r="J13" s="20">
         <f>SUM(I2:J11)</f>
-        <v>0</v>
+        <v>64.5</v>
       </c>
       <c r="K13" s="20"/>
       <c r="L13" s="20">
@@ -5741,23 +5771,23 @@
       </c>
       <c r="H14" s="18">
         <f t="shared" si="4"/>
-        <v>501.5</v>
+        <v>499.5</v>
       </c>
       <c r="I14" s="18">
         <f t="shared" si="4"/>
-        <v>501.5</v>
+        <v>435</v>
       </c>
       <c r="J14" s="18">
         <f t="shared" si="4"/>
-        <v>501.5</v>
+        <v>435</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="4"/>
-        <v>501.5</v>
+        <v>435</v>
       </c>
       <c r="L14" s="18">
         <f t="shared" si="4"/>
-        <v>501.5</v>
+        <v>435</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12075,16 +12105,20 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
+      <c r="A16" s="9" t="s">
+        <v>79</v>
+      </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="G16" s="10">
+        <v>1</v>
+      </c>
       <c r="H16" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -12140,11 +12174,11 @@
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -12244,10 +12278,12 @@
         <v>1</v>
       </c>
       <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
+      <c r="G25" s="10">
+        <v>1</v>
+      </c>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -12303,11 +12339,11 @@
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -13761,21 +13797,35 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="D5" s="10">
+        <v>1</v>
+      </c>
+      <c r="E5" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G5" s="10"/>
       <c r="H5" s="6">
         <f>SUM(B5:G5)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
+      <c r="A6" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="10">
+        <v>1</v>
+      </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
@@ -13783,12 +13833,16 @@
       <c r="G6" s="10"/>
       <c r="H6" s="6">
         <f t="shared" ref="H6:H9" si="0">SUM(B6:G6)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10"/>
+      <c r="A7" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="10">
+        <v>1</v>
+      </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
@@ -13796,7 +13850,7 @@
       <c r="G7" s="10"/>
       <c r="H7" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -13832,7 +13886,7 @@
       </c>
       <c r="B10" s="11">
         <f t="shared" ref="B10:G10" si="1">SUM(B5:B9)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="C10" s="11">
         <f t="shared" si="1"/>
@@ -13840,15 +13894,15 @@
       </c>
       <c r="D10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
@@ -13856,7 +13910,7 @@
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -13920,42 +13974,60 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="D14" s="10">
+        <v>1</v>
+      </c>
+      <c r="E14" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G14" s="10"/>
       <c r="H14" s="6">
         <f>SUM(B14:G14)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
+      <c r="A15" s="9" t="s">
+        <v>77</v>
+      </c>
       <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
+      <c r="C15" s="10">
+        <v>1</v>
+      </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="6">
         <f t="shared" ref="H15:H18" si="2">SUM(B15:G15)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
+      <c r="A16" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
+      <c r="E16" s="10">
+        <v>1</v>
+      </c>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -13991,23 +14063,23 @@
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:G19" si="3">SUM(B14:B18)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
@@ -14015,7 +14087,7 @@
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14069,55 +14141,79 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
+      <c r="D23" s="10">
+        <v>1</v>
+      </c>
       <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="F23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G23" s="10"/>
       <c r="H23" s="6">
         <f>SUM(B23:G23)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="9"/>
+      <c r="A24" s="9" t="s">
+        <v>75</v>
+      </c>
       <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
+      <c r="C24" s="10">
+        <v>1</v>
+      </c>
       <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
+      <c r="E24" s="10">
+        <v>0.5</v>
+      </c>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="6">
         <f t="shared" ref="H24:H27" si="4">SUM(B24:G24)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="9"/>
-      <c r="B25" s="10"/>
+      <c r="A25" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="10">
+        <v>1.5</v>
+      </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="10">
+        <v>0.5</v>
+      </c>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="9"/>
+      <c r="A26" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
+      <c r="E26" s="10">
+        <v>0.5</v>
+      </c>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
       <c r="H26" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -14140,23 +14236,23 @@
       </c>
       <c r="B28" s="11">
         <f t="shared" ref="B28:G28" si="5">SUM(B23:B27)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
@@ -14164,7 +14260,7 @@
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14218,16 +14314,22 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
+      <c r="A32" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="10">
+        <v>1.5</v>
+      </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="F32" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G32" s="10"/>
       <c r="H32" s="6">
         <f>SUM(B32:G32)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -14289,7 +14391,7 @@
       </c>
       <c r="B37" s="11">
         <f t="shared" ref="B37:G37" si="7">SUM(B32:B36)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="C37" s="11">
         <f t="shared" si="7"/>
@@ -14305,7 +14407,7 @@
       </c>
       <c r="F37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G37" s="11">
         <f t="shared" si="7"/>
@@ -14313,7 +14415,7 @@
       </c>
       <c r="H37" s="11">
         <f>SUM(B37:G37)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14368,30 +14470,38 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B41" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
+      <c r="F41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G41" s="10"/>
       <c r="H41" s="6">
         <f>SUM(B41:G41)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="9"/>
+      <c r="A42" s="9" t="s">
+        <v>82</v>
+      </c>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
+      <c r="E42" s="10">
+        <v>1.5</v>
+      </c>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
       <c r="H42" s="6">
         <f t="shared" ref="H42:H45" si="9">SUM(B42:G42)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -14440,7 +14550,7 @@
       </c>
       <c r="B46" s="11">
         <f t="shared" ref="B46:G46" si="10">SUM(B41:B45)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C46" s="11">
         <f t="shared" si="10"/>
@@ -14452,11 +14562,11 @@
       </c>
       <c r="E46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
@@ -14464,7 +14574,7 @@
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14519,30 +14629,40 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
+      <c r="D50" s="10">
+        <v>1</v>
+      </c>
       <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
+      <c r="F50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G50" s="10"/>
       <c r="H50" s="6">
         <f>SUM(B50:G50)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="9"/>
+      <c r="A51" s="9" t="s">
+        <v>81</v>
+      </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
       <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
+      <c r="E51" s="10">
+        <v>4</v>
+      </c>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
       <c r="H51" s="6">
         <f t="shared" ref="H51:H54" si="12">SUM(B51:G51)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
@@ -14591,7 +14711,7 @@
       </c>
       <c r="B55" s="11">
         <f t="shared" ref="B55:G55" si="13">SUM(B50:B54)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C55" s="11">
         <f t="shared" si="13"/>
@@ -14599,15 +14719,15 @@
       </c>
       <c r="D55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
@@ -14615,7 +14735,7 @@
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14670,30 +14790,40 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
+      <c r="D59" s="10">
+        <v>1</v>
+      </c>
       <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
+      <c r="F59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G59" s="10"/>
       <c r="H59" s="6">
         <f>SUM(B59:G59)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
+      <c r="A60" s="9" t="s">
+        <v>83</v>
+      </c>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
       <c r="D60" s="10"/>
       <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
+      <c r="F60" s="10">
+        <v>4</v>
+      </c>
       <c r="G60" s="10"/>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -14742,7 +14872,7 @@
       </c>
       <c r="B64" s="11">
         <f t="shared" ref="B64:G64" si="16">SUM(B59:B63)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C64" s="11">
         <f t="shared" si="16"/>
@@ -14750,7 +14880,7 @@
       </c>
       <c r="D64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E64" s="11">
         <f t="shared" si="16"/>
@@ -14758,7 +14888,7 @@
       </c>
       <c r="F64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
@@ -14766,7 +14896,7 @@
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14821,30 +14951,40 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C68" s="10"/>
-      <c r="D68" s="10"/>
+      <c r="D68" s="10">
+        <v>1</v>
+      </c>
       <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
+      <c r="F68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G68" s="10"/>
       <c r="H68" s="6">
         <f>SUM(B68:G68)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="9"/>
+      <c r="A69" s="9" t="s">
+        <v>84</v>
+      </c>
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
+      <c r="D69" s="10">
+        <v>1</v>
+      </c>
       <c r="E69" s="10"/>
       <c r="F69" s="10"/>
       <c r="G69" s="10"/>
       <c r="H69" s="6">
         <f t="shared" ref="H69:H72" si="18">SUM(B69:G69)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -14893,7 +15033,7 @@
       </c>
       <c r="B73" s="11">
         <f t="shared" ref="B73:G73" si="19">SUM(B68:B72)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C73" s="11">
         <f t="shared" si="19"/>
@@ -14901,7 +15041,7 @@
       </c>
       <c r="D73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E73" s="11">
         <f t="shared" si="19"/>
@@ -14909,7 +15049,7 @@
       </c>
       <c r="F73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
@@ -14917,7 +15057,7 @@
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update the hour log for week 6.
</commit_message>
<xml_diff>
--- a/docs/2.2_P.CoB_Time_registration_for10.xlsx
+++ b/docs/2.2_P.CoB_Time_registration_for10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shawn\Dev\ClientOnBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AE327A-F333-4DA9-8345-4621810C313F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB372C1-FEC0-47DF-B99D-DF7EA7807F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructie" sheetId="19" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="98">
   <si>
     <t>Kickoff</t>
   </si>
@@ -270,9 +270,6 @@
     <t>API request for modifying a user</t>
   </si>
   <si>
-    <t>Reviewing merge requests</t>
-  </si>
-  <si>
     <t>Adding nodes in editor</t>
   </si>
   <si>
@@ -298,6 +295,48 @@
   </si>
   <si>
     <t>API request for adding users to a session</t>
+  </si>
+  <si>
+    <t>Editing nodes in editor</t>
+  </si>
+  <si>
+    <t>Reviewing merge requests + providing help</t>
+  </si>
+  <si>
+    <t>Fixing issues with fetch wrapper</t>
+  </si>
+  <si>
+    <t>Editing edges in editor</t>
+  </si>
+  <si>
+    <t>Reviewing merge requests</t>
+  </si>
+  <si>
+    <t>Creating review action when adding a node</t>
+  </si>
+  <si>
+    <t>Fetching all review actions to the history bar (frontend)</t>
+  </si>
+  <si>
+    <t>Closing and opening sessions (frontend)</t>
+  </si>
+  <si>
+    <t>Setting up web sockets (fixing issues)</t>
+  </si>
+  <si>
+    <t>API request for getting a single past action</t>
+  </si>
+  <si>
+    <t>Learning socket.io</t>
+  </si>
+  <si>
+    <t>Automated testing for backend</t>
+  </si>
+  <si>
+    <t>API request for changing the status of sessions</t>
+  </si>
+  <si>
+    <t>Context research</t>
   </si>
 </sst>
 </file>
@@ -765,12 +804,6 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -779,6 +812,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -911,10 +950,10 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.5</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -997,10 +1036,10 @@
                   <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.5</c:v>
+                  <c:v>9.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1083,10 +1122,10 @@
                   <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1172,7 +1211,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1255,10 +1294,10 @@
                   <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.5</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1341,10 +1380,10 @@
                   <c:v>11.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1427,10 +1466,10 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1513,10 +1552,10 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -1924,16 +1963,16 @@
                   <c:v>499.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>435</c:v>
+                  <c:v>419</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>435</c:v>
+                  <c:v>353.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>435</c:v>
+                  <c:v>353.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>435</c:v>
+                  <c:v>353.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3472,32 +3511,32 @@
         <f>Total!$L$1</f>
         <v>Week 8</v>
       </c>
-      <c r="B1" s="40" t="str">
+      <c r="B1" s="43" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="str">
+      <c r="B3" s="40" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -3647,16 +3686,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="42" t="str">
+      <c r="B12" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -3796,16 +3835,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="42" t="str">
+      <c r="B21" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -3945,16 +3984,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="42" t="str">
+      <c r="B30" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -4094,16 +4133,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="42" t="str">
+      <c r="B39" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -4245,16 +4284,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="42" t="str">
+      <c r="B48" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="42"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -4396,16 +4435,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="42" t="str">
+      <c r="B57" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -4547,16 +4586,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="42" t="str">
+      <c r="B66" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="43"/>
-      <c r="D66" s="43"/>
-      <c r="E66" s="43"/>
-      <c r="F66" s="43"/>
-      <c r="G66" s="43"/>
-      <c r="H66" s="44"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="42"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -4698,16 +4737,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="42" t="str">
+      <c r="B75" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="43"/>
-      <c r="D75" s="43"/>
-      <c r="E75" s="43"/>
-      <c r="F75" s="43"/>
-      <c r="G75" s="43"/>
-      <c r="H75" s="44"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="42"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -4849,16 +4888,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="42" t="str">
+      <c r="B84" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="43"/>
-      <c r="D84" s="43"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="44"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="41"/>
+      <c r="F84" s="41"/>
+      <c r="G84" s="41"/>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -4997,17 +5036,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5279,11 +5318,11 @@
       </c>
       <c r="I2" s="3">
         <f>'Week (5)'!$H$10</f>
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="J2" s="3">
         <f>'Week (6)'!$H$10</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K2" s="3">
         <f>'Week (7)'!$H$10</f>
@@ -5295,7 +5334,7 @@
       </c>
       <c r="M2" s="4">
         <f>SUM(E2:L2)</f>
-        <v>36.5</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5322,11 +5361,11 @@
       </c>
       <c r="I3" s="3">
         <f>'Week (5)'!$H$19</f>
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="J3" s="3">
         <f>'Week (6)'!$H$19</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="K3" s="3">
         <f>'Week (7)'!$H$19</f>
@@ -5338,7 +5377,7 @@
       </c>
       <c r="M3" s="4">
         <f t="shared" ref="M3:M5" si="0">SUM(E3:L3)</f>
-        <v>41</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5369,11 +5408,11 @@
       </c>
       <c r="I4" s="3">
         <f>'Week (5)'!$H$28</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J4" s="3">
         <f>'Week (6)'!$H$28</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="K4" s="3">
         <f>'Week (7)'!$H$28</f>
@@ -5385,7 +5424,7 @@
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>68.5</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -5416,7 +5455,7 @@
       </c>
       <c r="J5" s="3">
         <f>'Week (6)'!$H$37</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K5" s="3">
         <f>'Week (7)'!$H$37</f>
@@ -5428,7 +5467,7 @@
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5455,11 +5494,11 @@
       </c>
       <c r="I6" s="3">
         <f>'Week (5)'!$H$46</f>
-        <v>6.5</v>
+        <v>8.5</v>
       </c>
       <c r="J6" s="3">
         <f>'Week (6)'!$H$46</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K6" s="3">
         <f>'Week (7)'!$H$46</f>
@@ -5471,7 +5510,7 @@
       </c>
       <c r="M6" s="4">
         <f t="shared" ref="M6" si="1">SUM(E6:L6)</f>
-        <v>49</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5498,11 +5537,11 @@
       </c>
       <c r="I7" s="3">
         <f>'Week (5)'!$H$55</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="J7" s="3">
         <f>'Week (6)'!$H$55</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="K7" s="3">
         <f>'Week (7)'!$H$55</f>
@@ -5514,7 +5553,7 @@
       </c>
       <c r="M7" s="4">
         <f t="shared" ref="M7:M11" si="2">SUM(E7:L7)</f>
-        <v>48.5</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5541,11 +5580,11 @@
       </c>
       <c r="I8" s="3">
         <f>'Week (5)'!$H$64</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J8" s="3">
         <f>'Week (6)'!$H$64</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K8" s="3">
         <f>'Week (7)'!$H$64</f>
@@ -5557,7 +5596,7 @@
       </c>
       <c r="M8" s="4">
         <f t="shared" si="2"/>
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5584,11 +5623,11 @@
       </c>
       <c r="I9" s="3">
         <f>'Week (5)'!$H$73</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J9" s="3">
         <f>'Week (6)'!$H$73</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K9" s="3">
         <f>'Week (7)'!$H$73</f>
@@ -5600,7 +5639,7 @@
       </c>
       <c r="M9" s="4">
         <f t="shared" si="2"/>
-        <v>29</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5709,11 +5748,11 @@
       </c>
       <c r="I12" s="15">
         <f t="shared" si="3"/>
-        <v>64.5</v>
+        <v>80.5</v>
       </c>
       <c r="J12" s="15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>65.5</v>
       </c>
       <c r="K12" s="15">
         <f t="shared" si="3"/>
@@ -5743,7 +5782,7 @@
       <c r="I13" s="20"/>
       <c r="J13" s="20">
         <f>SUM(I2:J11)</f>
-        <v>64.5</v>
+        <v>146</v>
       </c>
       <c r="K13" s="20"/>
       <c r="L13" s="20">
@@ -5775,19 +5814,19 @@
       </c>
       <c r="I14" s="18">
         <f t="shared" si="4"/>
-        <v>435</v>
+        <v>419</v>
       </c>
       <c r="J14" s="18">
         <f t="shared" si="4"/>
-        <v>435</v>
+        <v>353.5</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="4"/>
-        <v>435</v>
+        <v>353.5</v>
       </c>
       <c r="L14" s="18">
         <f t="shared" si="4"/>
-        <v>435</v>
+        <v>353.5</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6121,30 +6160,30 @@
         <f>Total!$E$1</f>
         <v>Week 1</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
@@ -6307,16 +6346,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B13" s="42" t="str">
+      <c r="B13" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="42"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="str">
@@ -6467,16 +6506,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B23" s="42" t="str">
+      <c r="B23" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="44"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="42"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="str">
@@ -6626,16 +6665,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B32" s="42" t="str">
+      <c r="B32" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="44"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="42"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="str">
@@ -6783,16 +6822,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B41" s="42" t="str">
+      <c r="B41" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C41" s="43"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="43"/>
-      <c r="H41" s="44"/>
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="42"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="str">
@@ -6942,16 +6981,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B50" s="42" t="str">
+      <c r="B50" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C50" s="43"/>
-      <c r="D50" s="43"/>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="44"/>
+      <c r="C50" s="41"/>
+      <c r="D50" s="41"/>
+      <c r="E50" s="41"/>
+      <c r="F50" s="41"/>
+      <c r="G50" s="41"/>
+      <c r="H50" s="42"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="str">
@@ -7101,16 +7140,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B59" s="42" t="str">
+      <c r="B59" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C59" s="43"/>
-      <c r="D59" s="43"/>
-      <c r="E59" s="43"/>
-      <c r="F59" s="43"/>
-      <c r="G59" s="43"/>
-      <c r="H59" s="44"/>
+      <c r="C59" s="41"/>
+      <c r="D59" s="41"/>
+      <c r="E59" s="41"/>
+      <c r="F59" s="41"/>
+      <c r="G59" s="41"/>
+      <c r="H59" s="42"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="str">
@@ -7256,16 +7295,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B68" s="42" t="str">
+      <c r="B68" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C68" s="43"/>
-      <c r="D68" s="43"/>
-      <c r="E68" s="43"/>
-      <c r="F68" s="43"/>
-      <c r="G68" s="43"/>
-      <c r="H68" s="44"/>
+      <c r="C68" s="41"/>
+      <c r="D68" s="41"/>
+      <c r="E68" s="41"/>
+      <c r="F68" s="41"/>
+      <c r="G68" s="41"/>
+      <c r="H68" s="42"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="str">
@@ -7411,16 +7450,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B77" s="42" t="str">
+      <c r="B77" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C77" s="43"/>
-      <c r="D77" s="43"/>
-      <c r="E77" s="43"/>
-      <c r="F77" s="43"/>
-      <c r="G77" s="43"/>
-      <c r="H77" s="44"/>
+      <c r="C77" s="41"/>
+      <c r="D77" s="41"/>
+      <c r="E77" s="41"/>
+      <c r="F77" s="41"/>
+      <c r="G77" s="41"/>
+      <c r="H77" s="42"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="str">
@@ -7562,16 +7601,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B86" s="42" t="str">
+      <c r="B86" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C86" s="43"/>
-      <c r="D86" s="43"/>
-      <c r="E86" s="43"/>
-      <c r="F86" s="43"/>
-      <c r="G86" s="43"/>
-      <c r="H86" s="44"/>
+      <c r="C86" s="41"/>
+      <c r="D86" s="41"/>
+      <c r="E86" s="41"/>
+      <c r="F86" s="41"/>
+      <c r="G86" s="41"/>
+      <c r="H86" s="42"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="str">
@@ -7710,17 +7749,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B32:H32"/>
     <mergeCell ref="B86:H86"/>
     <mergeCell ref="B41:H41"/>
     <mergeCell ref="B50:H50"/>
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B68:H68"/>
     <mergeCell ref="B77:H77"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B32:H32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -8000,32 +8039,32 @@
         <f>Total!$F$1</f>
         <v>Week 2</v>
       </c>
-      <c r="B1" s="40" t="str">
+      <c r="B1" s="43" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="str">
+      <c r="B3" s="40" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -8183,16 +8222,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="42" t="str">
+      <c r="B12" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -8346,16 +8385,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="42" t="str">
+      <c r="B21" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -8523,16 +8562,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="42" t="str">
+      <c r="B30" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -8684,16 +8723,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="42" t="str">
+      <c r="B39" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -8849,16 +8888,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="42" t="str">
+      <c r="B48" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="42"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -9012,16 +9051,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="42" t="str">
+      <c r="B57" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -9171,16 +9210,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="42" t="str">
+      <c r="B66" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="43"/>
-      <c r="D66" s="43"/>
-      <c r="E66" s="43"/>
-      <c r="F66" s="43"/>
-      <c r="G66" s="43"/>
-      <c r="H66" s="44"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="42"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -9324,16 +9363,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="42" t="str">
+      <c r="B75" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="43"/>
-      <c r="D75" s="43"/>
-      <c r="E75" s="43"/>
-      <c r="F75" s="43"/>
-      <c r="G75" s="43"/>
-      <c r="H75" s="44"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="42"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -9475,16 +9514,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="42" t="str">
+      <c r="B84" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="43"/>
-      <c r="D84" s="43"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="44"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="41"/>
+      <c r="F84" s="41"/>
+      <c r="G84" s="41"/>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -9623,17 +9662,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9908,32 +9947,32 @@
         <f>Total!$G$1</f>
         <v>Week 3</v>
       </c>
-      <c r="B1" s="40" t="str">
+      <c r="B1" s="43" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="str">
+      <c r="B3" s="40" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -10099,16 +10138,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="42" t="str">
+      <c r="B12" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -10266,16 +10305,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="42" t="str">
+      <c r="B21" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -10433,16 +10472,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="42" t="str">
+      <c r="B30" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -10596,16 +10635,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="42" t="str">
+      <c r="B39" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -10767,16 +10806,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="42" t="str">
+      <c r="B48" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="42"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -10934,16 +10973,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="42" t="str">
+      <c r="B57" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -11095,16 +11134,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="42" t="str">
+      <c r="B66" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="43"/>
-      <c r="D66" s="43"/>
-      <c r="E66" s="43"/>
-      <c r="F66" s="43"/>
-      <c r="G66" s="43"/>
-      <c r="H66" s="44"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="42"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -11254,16 +11293,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="42" t="str">
+      <c r="B75" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="43"/>
-      <c r="D75" s="43"/>
-      <c r="E75" s="43"/>
-      <c r="F75" s="43"/>
-      <c r="G75" s="43"/>
-      <c r="H75" s="44"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="42"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -11405,16 +11444,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="42" t="str">
+      <c r="B84" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="43"/>
-      <c r="D84" s="43"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="44"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="41"/>
+      <c r="F84" s="41"/>
+      <c r="G84" s="41"/>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -11553,17 +11592,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -11838,32 +11877,32 @@
         <f>Total!$H$1</f>
         <v>Week 4</v>
       </c>
-      <c r="B1" s="40" t="str">
+      <c r="B1" s="43" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="str">
+      <c r="B3" s="40" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -12023,16 +12062,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="42" t="str">
+      <c r="B12" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -12106,7 +12145,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -12186,16 +12225,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="42" t="str">
+      <c r="B21" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -12351,16 +12390,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="42" t="str">
+      <c r="B30" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -12510,16 +12549,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="42" t="str">
+      <c r="B39" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -12671,16 +12710,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="42" t="str">
+      <c r="B48" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="42"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -12834,16 +12873,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="42" t="str">
+      <c r="B57" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -12993,16 +13032,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="42" t="str">
+      <c r="B66" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="43"/>
-      <c r="D66" s="43"/>
-      <c r="E66" s="43"/>
-      <c r="F66" s="43"/>
-      <c r="G66" s="43"/>
-      <c r="H66" s="44"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="42"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -13152,16 +13191,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="42" t="str">
+      <c r="B75" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="43"/>
-      <c r="D75" s="43"/>
-      <c r="E75" s="43"/>
-      <c r="F75" s="43"/>
-      <c r="G75" s="43"/>
-      <c r="H75" s="44"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="42"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -13303,16 +13342,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="42" t="str">
+      <c r="B84" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="43"/>
-      <c r="D84" s="43"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="44"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="41"/>
+      <c r="F84" s="41"/>
+      <c r="G84" s="41"/>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -13451,17 +13490,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -13736,31 +13775,31 @@
         <f>Total!$I$1</f>
         <v>Week 5</v>
       </c>
-      <c r="B1" s="40" t="str">
+      <c r="B1" s="43" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -13838,7 +13877,7 @@
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" s="10">
         <v>1</v>
@@ -13854,16 +13893,20 @@
       </c>
     </row>
     <row r="8" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="9"/>
+      <c r="A8" s="9" t="s">
+        <v>89</v>
+      </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
+      <c r="G8" s="10">
+        <v>2</v>
+      </c>
       <c r="H8" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -13906,11 +13949,11 @@
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -13928,16 +13971,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="42" t="str">
+      <c r="B12" s="40" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -13998,7 +14041,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10">
@@ -14015,7 +14058,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -14031,16 +14074,20 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="9"/>
+      <c r="A17" s="9" t="s">
+        <v>93</v>
+      </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10">
+        <v>1</v>
+      </c>
       <c r="H17" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -14083,11 +14130,11 @@
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14095,16 +14142,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="42" t="str">
+      <c r="B21" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -14163,7 +14210,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="10">
@@ -14173,16 +14220,20 @@
       <c r="E24" s="10">
         <v>0.5</v>
       </c>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
+      <c r="F24" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="G24" s="10">
+        <v>1</v>
+      </c>
       <c r="H24" s="6">
         <f t="shared" ref="H24:H27" si="4">SUM(B24:G24)</f>
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B25" s="10">
         <v>1.5</v>
@@ -14217,16 +14268,20 @@
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="9"/>
+      <c r="A27" s="9" t="s">
+        <v>84</v>
+      </c>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10">
+        <v>3.5</v>
+      </c>
       <c r="H27" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="22" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -14252,15 +14307,15 @@
       </c>
       <c r="F28" s="11">
         <f t="shared" si="5"/>
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14268,16 +14323,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="42" t="str">
+      <c r="B30" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -14423,16 +14478,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="42" t="str">
+      <c r="B39" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -14489,7 +14544,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
@@ -14498,10 +14553,12 @@
         <v>1.5</v>
       </c>
       <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
+      <c r="G42" s="10">
+        <v>2</v>
+      </c>
       <c r="H42" s="6">
         <f t="shared" ref="H42:H45" si="9">SUM(B42:G42)</f>
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -14570,11 +14627,11 @@
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>6.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14582,16 +14639,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="42" t="str">
+      <c r="B48" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="42"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -14650,7 +14707,7 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
@@ -14659,10 +14716,12 @@
         <v>4</v>
       </c>
       <c r="F51" s="10"/>
-      <c r="G51" s="10"/>
+      <c r="G51" s="10">
+        <v>4</v>
+      </c>
       <c r="H51" s="6">
         <f t="shared" ref="H51:H54" si="12">SUM(B51:G51)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
@@ -14731,11 +14790,11 @@
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14743,16 +14802,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="42" t="str">
+      <c r="B57" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -14811,7 +14870,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
@@ -14820,10 +14879,12 @@
       <c r="F60" s="10">
         <v>4</v>
       </c>
-      <c r="G60" s="10"/>
+      <c r="G60" s="10">
+        <v>1</v>
+      </c>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -14892,11 +14953,11 @@
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -14904,16 +14965,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="42" t="str">
+      <c r="B66" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="43"/>
-      <c r="D66" s="43"/>
-      <c r="E66" s="43"/>
-      <c r="F66" s="43"/>
-      <c r="G66" s="43"/>
-      <c r="H66" s="44"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="42"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -14972,7 +15033,7 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
@@ -14988,16 +15049,20 @@
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" s="9"/>
+      <c r="A70" s="9" t="s">
+        <v>96</v>
+      </c>
       <c r="B70" s="10"/>
       <c r="C70" s="10"/>
       <c r="D70" s="10"/>
       <c r="E70" s="10"/>
       <c r="F70" s="10"/>
-      <c r="G70" s="10"/>
+      <c r="G70" s="10">
+        <v>1</v>
+      </c>
       <c r="H70" s="6">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
@@ -15053,11 +15118,11 @@
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -15065,16 +15130,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="42" t="str">
+      <c r="B75" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="43"/>
-      <c r="D75" s="43"/>
-      <c r="E75" s="43"/>
-      <c r="F75" s="43"/>
-      <c r="G75" s="43"/>
-      <c r="H75" s="44"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="42"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -15216,16 +15281,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="42" t="str">
+      <c r="B84" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="43"/>
-      <c r="D84" s="43"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="44"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="41"/>
+      <c r="F84" s="41"/>
+      <c r="G84" s="41"/>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -15364,17 +15429,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -15649,32 +15714,32 @@
         <f>Total!$J$1</f>
         <v>Week 6</v>
       </c>
-      <c r="B1" s="40" t="str">
+      <c r="B1" s="43" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="str">
+      <c r="B3" s="40" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -15711,42 +15776,58 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G5" s="10"/>
       <c r="H5" s="6">
         <f>SUM(B5:G5)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
+      <c r="A6" s="9" t="s">
+        <v>90</v>
+      </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="E6" s="10">
+        <v>1</v>
+      </c>
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="6">
         <f t="shared" ref="H6:H9" si="0">SUM(B6:G6)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="9"/>
+      <c r="A7" s="9" t="s">
+        <v>88</v>
+      </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
+      <c r="E7" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="F7" s="10">
+        <v>0.5</v>
+      </c>
       <c r="G7" s="10"/>
       <c r="H7" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -15782,7 +15863,7 @@
       </c>
       <c r="B10" s="11">
         <f t="shared" ref="B10:G10" si="1">SUM(B5:B9)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C10" s="11">
         <f t="shared" si="1"/>
@@ -15794,11 +15875,11 @@
       </c>
       <c r="E10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
@@ -15806,7 +15887,7 @@
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -15824,16 +15905,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="42" t="str">
+      <c r="B12" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -15870,42 +15951,56 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="F14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G14" s="10"/>
       <c r="H14" s="6">
         <f>SUM(B14:G14)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
+      <c r="A15" s="9" t="s">
+        <v>88</v>
+      </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
+      <c r="E15" s="10">
+        <v>0.5</v>
+      </c>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="6">
         <f t="shared" ref="H15:H18" si="2">SUM(B15:G15)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
+      <c r="A16" s="9" t="s">
+        <v>94</v>
+      </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
+      <c r="E16" s="10">
+        <v>1</v>
+      </c>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -15941,7 +16036,7 @@
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:G19" si="3">SUM(B14:B18)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="3"/>
@@ -15953,11 +16048,11 @@
       </c>
       <c r="E19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
@@ -15965,7 +16060,7 @@
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -15973,16 +16068,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="42" t="str">
+      <c r="B21" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -16019,55 +16114,73 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="F23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G23" s="10"/>
       <c r="H23" s="6">
         <f>SUM(B23:G23)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="9"/>
+      <c r="A24" s="9" t="s">
+        <v>86</v>
+      </c>
       <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
+      <c r="C24" s="10">
+        <v>0.5</v>
+      </c>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="6">
         <f t="shared" ref="H24:H27" si="4">SUM(B24:G24)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="9"/>
+      <c r="A25" s="9" t="s">
+        <v>87</v>
+      </c>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="10">
+        <v>2.5</v>
+      </c>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="9"/>
+      <c r="A26" s="9" t="s">
+        <v>88</v>
+      </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
+      <c r="E26" s="10">
+        <v>0.5</v>
+      </c>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
       <c r="H26" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -16090,11 +16203,11 @@
       </c>
       <c r="B28" s="11">
         <f t="shared" ref="B28:G28" si="5">SUM(B23:B27)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D28" s="11">
         <f t="shared" si="5"/>
@@ -16102,11 +16215,11 @@
       </c>
       <c r="E28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
@@ -16114,7 +16227,7 @@
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16122,16 +16235,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="42" t="str">
+      <c r="B30" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -16168,29 +16281,39 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
+      <c r="A32" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="10">
+        <v>1.5</v>
+      </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="F32" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G32" s="10"/>
       <c r="H32" s="6">
         <f>SUM(B32:G32)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="9"/>
+      <c r="A33" s="9" t="s">
+        <v>95</v>
+      </c>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
+      <c r="E33" s="10">
+        <v>3</v>
+      </c>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
       <c r="H33" s="6">
         <f t="shared" ref="H33:H36" si="6">SUM(B33:G33)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -16239,7 +16362,7 @@
       </c>
       <c r="B37" s="11">
         <f t="shared" ref="B37:G37" si="7">SUM(B32:B36)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="C37" s="11">
         <f t="shared" si="7"/>
@@ -16251,11 +16374,11 @@
       </c>
       <c r="E37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G37" s="11">
         <f t="shared" si="7"/>
@@ -16263,7 +16386,7 @@
       </c>
       <c r="H37" s="11">
         <f>SUM(B37:G37)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16271,23 +16394,26 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="42" t="str">
+      <c r="B39" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
         <f>$A$4</f>
         <v>User story / task description</v>
       </c>
-      <c r="B40" s="8"/>
+      <c r="B40" s="8" t="str">
+        <f>'Week (1)'!B$4</f>
+        <v>Ma</v>
+      </c>
       <c r="C40" s="8" t="str">
         <f t="shared" ref="C40:H40" si="8">C$4</f>
         <v>Di</v>
@@ -16315,43 +16441,57 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B41" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
+      <c r="F41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G41" s="10"/>
       <c r="H41" s="6">
         <f>SUM(B41:G41)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="9"/>
+      <c r="A42" s="9" t="s">
+        <v>91</v>
+      </c>
       <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
+      <c r="C42" s="10">
+        <v>1</v>
+      </c>
+      <c r="D42" s="10">
+        <v>2</v>
+      </c>
       <c r="E42" s="10"/>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
       <c r="H42" s="6">
         <f t="shared" ref="H42:H45" si="9">SUM(B42:G42)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="9"/>
+      <c r="A43" s="9" t="s">
+        <v>88</v>
+      </c>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
+      <c r="D43" s="10">
+        <v>1</v>
+      </c>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
       <c r="H43" s="6">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -16387,15 +16527,15 @@
       </c>
       <c r="B46" s="11">
         <f t="shared" ref="B46:G46" si="10">SUM(B41:B45)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E46" s="11">
         <f t="shared" si="10"/>
@@ -16403,7 +16543,7 @@
       </c>
       <c r="F46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
@@ -16411,7 +16551,7 @@
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16419,16 +16559,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="42" t="str">
+      <c r="B48" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="42"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -16466,30 +16606,38 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
+      <c r="F50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G50" s="10"/>
       <c r="H50" s="6">
         <f>SUM(B50:G50)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="9"/>
+      <c r="A51" s="9" t="s">
+        <v>92</v>
+      </c>
       <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
+      <c r="C51" s="10">
+        <v>1.5</v>
+      </c>
       <c r="D51" s="10"/>
       <c r="E51" s="10"/>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
       <c r="H51" s="6">
         <f t="shared" ref="H51:H54" si="12">SUM(B51:G51)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
@@ -16538,11 +16686,11 @@
       </c>
       <c r="B55" s="11">
         <f t="shared" ref="B55:G55" si="13">SUM(B50:B54)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="D55" s="11">
         <f t="shared" si="13"/>
@@ -16554,7 +16702,7 @@
       </c>
       <c r="F55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
@@ -16562,7 +16710,7 @@
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16570,16 +16718,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="42" t="str">
+      <c r="B57" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -16617,30 +16765,38 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
+      <c r="F59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G59" s="10"/>
       <c r="H59" s="6">
         <f>SUM(B59:G59)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
+      <c r="A60" s="9" t="s">
+        <v>82</v>
+      </c>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
       <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
+      <c r="E60" s="10">
+        <v>4</v>
+      </c>
       <c r="F60" s="10"/>
       <c r="G60" s="10"/>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -16689,7 +16845,7 @@
       </c>
       <c r="B64" s="11">
         <f t="shared" ref="B64:G64" si="16">SUM(B59:B63)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C64" s="11">
         <f t="shared" si="16"/>
@@ -16701,11 +16857,11 @@
       </c>
       <c r="E64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
@@ -16713,7 +16869,7 @@
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16721,16 +16877,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="42" t="str">
+      <c r="B66" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="43"/>
-      <c r="D66" s="43"/>
-      <c r="E66" s="43"/>
-      <c r="F66" s="43"/>
-      <c r="G66" s="43"/>
-      <c r="H66" s="44"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="42"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -16768,30 +16924,40 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
+      <c r="F68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G68" s="10"/>
       <c r="H68" s="6">
         <f>SUM(B68:G68)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="9"/>
-      <c r="B69" s="10"/>
+      <c r="A69" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69" s="10">
+        <v>4</v>
+      </c>
       <c r="C69" s="10"/>
       <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
+      <c r="E69" s="10">
+        <v>3</v>
+      </c>
       <c r="F69" s="10"/>
       <c r="G69" s="10"/>
       <c r="H69" s="6">
         <f t="shared" ref="H69:H72" si="18">SUM(B69:G69)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -16840,7 +17006,7 @@
       </c>
       <c r="B73" s="11">
         <f t="shared" ref="B73:G73" si="19">SUM(B68:B72)</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="C73" s="11">
         <f t="shared" si="19"/>
@@ -16852,11 +17018,11 @@
       </c>
       <c r="E73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
@@ -16864,7 +17030,7 @@
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16872,16 +17038,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="42" t="str">
+      <c r="B75" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="43"/>
-      <c r="D75" s="43"/>
-      <c r="E75" s="43"/>
-      <c r="F75" s="43"/>
-      <c r="G75" s="43"/>
-      <c r="H75" s="44"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="42"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -17023,16 +17189,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="42" t="str">
+      <c r="B84" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="43"/>
-      <c r="D84" s="43"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="44"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="41"/>
+      <c r="F84" s="41"/>
+      <c r="G84" s="41"/>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -17171,17 +17337,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -17456,32 +17622,32 @@
         <f>Total!$K$1</f>
         <v>Week 7</v>
       </c>
-      <c r="B1" s="40" t="str">
+      <c r="B1" s="43" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="41"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="42" t="str">
+      <c r="B3" s="40" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -17631,16 +17797,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="42" t="str">
+      <c r="B12" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -17780,16 +17946,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="42" t="str">
+      <c r="B21" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -17929,16 +18095,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="42" t="str">
+      <c r="B30" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41"/>
+      <c r="H30" s="42"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -18078,16 +18244,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="42" t="str">
+      <c r="B39" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="42"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -18229,16 +18395,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="42" t="str">
+      <c r="B48" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="43"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="42"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -18380,16 +18546,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="42" t="str">
+      <c r="B57" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="41"/>
+      <c r="H57" s="42"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -18531,16 +18697,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="42" t="str">
+      <c r="B66" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="43"/>
-      <c r="D66" s="43"/>
-      <c r="E66" s="43"/>
-      <c r="F66" s="43"/>
-      <c r="G66" s="43"/>
-      <c r="H66" s="44"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="42"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -18682,16 +18848,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="42" t="str">
+      <c r="B75" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="43"/>
-      <c r="D75" s="43"/>
-      <c r="E75" s="43"/>
-      <c r="F75" s="43"/>
-      <c r="G75" s="43"/>
-      <c r="H75" s="44"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="42"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -18833,16 +18999,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="42" t="str">
+      <c r="B84" s="40" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="43"/>
-      <c r="D84" s="43"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="44"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="41"/>
+      <c r="F84" s="41"/>
+      <c r="G84" s="41"/>
+      <c r="H84" s="42"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -18981,17 +19147,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -18999,6 +19165,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <c6664f9864b54a78bdf9e6230de1c78b xmlns="6c73e52c-07d4-4617-ab67-464747257e8d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </c6664f9864b54a78bdf9e6230de1c78b>
+    <Versiebeheer xmlns="ab37b2fe-4f81-426e-b942-40459dbac68c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100294690D6A57C3C4B8650464765815F1C" ma:contentTypeVersion="15" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="bf1d2ff51e740e451b46e7c13bf9e6da">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="45f6ce90-ba85-4ef2-b43f-c64448cd95eb" xmlns:ns3="c7549584-aa9c-449c-abfe-2ca02f3a7188" xmlns:ns4="6c73e52c-07d4-4617-ab67-464747257e8d" xmlns:ns5="ab37b2fe-4f81-426e-b942-40459dbac68c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8575fd65d7959dd12bd4dc11d36e634e" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="45f6ce90-ba85-4ef2-b43f-c64448cd95eb"/>
@@ -19241,27 +19427,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <c6664f9864b54a78bdf9e6230de1c78b xmlns="6c73e52c-07d4-4617-ab67-464747257e8d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </c6664f9864b54a78bdf9e6230de1c78b>
-    <Versiebeheer xmlns="ab37b2fe-4f81-426e-b942-40459dbac68c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{844B94A5-2CB8-4D3A-A97F-85854BBCA257}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477D1558-F7E0-401F-8472-E1151A96BE17}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c73e52c-07d4-4617-ab67-464747257e8d"/>
+    <ds:schemaRef ds:uri="ab37b2fe-4f81-426e-b942-40459dbac68c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{724CCB8E-5E6A-4B8C-A558-5D9223ADF390}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19280,23 +19465,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477D1558-F7E0-401F-8472-E1151A96BE17}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c73e52c-07d4-4617-ab67-464747257e8d"/>
-    <ds:schemaRef ds:uri="ab37b2fe-4f81-426e-b942-40459dbac68c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{844B94A5-2CB8-4D3A-A97F-85854BBCA257}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the hour log for the week 7.
</commit_message>
<xml_diff>
--- a/docs/2.2_P.CoB_Time_registration_for10.xlsx
+++ b/docs/2.2_P.CoB_Time_registration_for10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shawn\Dev\ClientOnBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB372C1-FEC0-47DF-B99D-DF7EA7807F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6518D0F2-3554-44C2-BA4D-D03CC9C562E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructie" sheetId="19" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="110">
   <si>
     <t>Kickoff</t>
   </si>
@@ -337,6 +337,42 @@
   </si>
   <si>
     <t>Context research</t>
+  </si>
+  <si>
+    <t>Deleting elements in the editor</t>
+  </si>
+  <si>
+    <t>Documenting the second meeting with the client</t>
+  </si>
+  <si>
+    <t>Documentation of problem analysis and alternatives</t>
+  </si>
+  <si>
+    <t>Backend for deleting users</t>
+  </si>
+  <si>
+    <t>Creating API endpoint for inviteable members</t>
+  </si>
+  <si>
+    <t>Streaming cursors of users in the editor</t>
+  </si>
+  <si>
+    <t>Helping teammates</t>
+  </si>
+  <si>
+    <t>History bar</t>
+  </si>
+  <si>
+    <t>Frontend page for creating a session</t>
+  </si>
+  <si>
+    <t>Documentation of Socket.IO</t>
+  </si>
+  <si>
+    <t>Display the history state of the editor</t>
+  </si>
+  <si>
+    <t>Rendering the list of history entries in the action bar</t>
   </si>
 </sst>
 </file>
@@ -804,6 +840,12 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -812,12 +854,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -953,10 +989,10 @@
                   <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1039,10 +1075,10 @@
                   <c:v>9.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6.5</c:v>
+                  <c:v>9.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1128,7 +1164,7 @@
                   <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>9.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1211,10 +1247,10 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1300,7 +1336,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1386,7 +1422,7 @@
                   <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1472,7 +1508,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>13.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1558,7 +1594,7 @@
                   <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>3.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1966,13 +2002,13 @@
                   <c:v>419</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>353.5</c:v>
+                  <c:v>345.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>353.5</c:v>
+                  <c:v>284.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>353.5</c:v>
+                  <c:v>284.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3511,32 +3547,32 @@
         <f>Total!$L$1</f>
         <v>Week 8</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -3686,16 +3722,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -3835,16 +3871,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -3984,16 +4020,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -4133,16 +4169,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -4284,16 +4320,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -4435,16 +4471,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -4586,16 +4622,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="40" t="str">
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -4737,16 +4773,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -4888,16 +4924,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -5036,17 +5072,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5322,11 +5358,11 @@
       </c>
       <c r="J2" s="3">
         <f>'Week (6)'!$H$10</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K2" s="3">
         <f>'Week (7)'!$H$10</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L2" s="3">
         <f>'Week (8)'!$H$10</f>
@@ -5334,7 +5370,7 @@
       </c>
       <c r="M2" s="4">
         <f>SUM(E2:L2)</f>
-        <v>45.5</v>
+        <v>53.5</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5365,11 +5401,11 @@
       </c>
       <c r="J3" s="3">
         <f>'Week (6)'!$H$19</f>
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
       <c r="K3" s="3">
         <f>'Week (7)'!$H$19</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L3" s="3">
         <f>'Week (8)'!$H$19</f>
@@ -5377,7 +5413,7 @@
       </c>
       <c r="M3" s="4">
         <f t="shared" ref="M3:M5" si="0">SUM(E3:L3)</f>
-        <v>48.5</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5416,7 +5452,7 @@
       </c>
       <c r="K4" s="3">
         <f>'Week (7)'!$H$28</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="L4" s="3">
         <f>'Week (8)'!$H$28</f>
@@ -5424,7 +5460,7 @@
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>68.5</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -5455,11 +5491,11 @@
       </c>
       <c r="J5" s="3">
         <f>'Week (6)'!$H$37</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K5" s="3">
         <f>'Week (7)'!$H$37</f>
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="L5" s="3">
         <f>'Week (8)'!$H$37</f>
@@ -5467,7 +5503,7 @@
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5502,7 +5538,7 @@
       </c>
       <c r="K6" s="3">
         <f>'Week (7)'!$H$46</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L6" s="3">
         <f>'Week (8)'!$H$46</f>
@@ -5510,7 +5546,7 @@
       </c>
       <c r="M6" s="4">
         <f t="shared" ref="M6" si="1">SUM(E6:L6)</f>
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5545,7 +5581,7 @@
       </c>
       <c r="K7" s="3">
         <f>'Week (7)'!$H$55</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L7" s="3">
         <f>'Week (8)'!$H$55</f>
@@ -5553,7 +5589,7 @@
       </c>
       <c r="M7" s="4">
         <f t="shared" ref="M7:M11" si="2">SUM(E7:L7)</f>
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5588,7 +5624,7 @@
       </c>
       <c r="K8" s="3">
         <f>'Week (7)'!$H$64</f>
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="L8" s="3">
         <f>'Week (8)'!$H$64</f>
@@ -5596,7 +5632,7 @@
       </c>
       <c r="M8" s="4">
         <f t="shared" si="2"/>
-        <v>51</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5631,7 +5667,7 @@
       </c>
       <c r="K9" s="3">
         <f>'Week (7)'!$H$73</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="L9" s="3">
         <f>'Week (8)'!$H$73</f>
@@ -5639,7 +5675,7 @@
       </c>
       <c r="M9" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5752,11 +5788,11 @@
       </c>
       <c r="J12" s="15">
         <f t="shared" si="3"/>
-        <v>65.5</v>
+        <v>73.5</v>
       </c>
       <c r="K12" s="15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="L12" s="15">
         <f t="shared" si="3"/>
@@ -5782,12 +5818,12 @@
       <c r="I13" s="20"/>
       <c r="J13" s="20">
         <f>SUM(I2:J11)</f>
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K13" s="20"/>
       <c r="L13" s="20">
         <f>SUM(K12:L12)</f>
-        <v>0</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5818,15 +5854,15 @@
       </c>
       <c r="J14" s="18">
         <f t="shared" si="4"/>
-        <v>353.5</v>
+        <v>345.5</v>
       </c>
       <c r="K14" s="18">
         <f t="shared" si="4"/>
-        <v>353.5</v>
+        <v>284.5</v>
       </c>
       <c r="L14" s="18">
         <f t="shared" si="4"/>
-        <v>353.5</v>
+        <v>284.5</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6160,30 +6196,30 @@
         <f>Total!$E$1</f>
         <v>Week 1</v>
       </c>
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
@@ -6346,16 +6382,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B13" s="40" t="str">
+      <c r="B13" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C13" s="41"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="44"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="str">
@@ -6506,16 +6542,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B23" s="40" t="str">
+      <c r="B23" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="42"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="44"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="str">
@@ -6665,16 +6701,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B32" s="40" t="str">
+      <c r="B32" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C32" s="41"/>
-      <c r="D32" s="41"/>
-      <c r="E32" s="41"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="41"/>
-      <c r="H32" s="42"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="43"/>
+      <c r="H32" s="44"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="str">
@@ -6822,16 +6858,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B41" s="40" t="str">
+      <c r="B41" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C41" s="41"/>
-      <c r="D41" s="41"/>
-      <c r="E41" s="41"/>
-      <c r="F41" s="41"/>
-      <c r="G41" s="41"/>
-      <c r="H41" s="42"/>
+      <c r="C41" s="43"/>
+      <c r="D41" s="43"/>
+      <c r="E41" s="43"/>
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+      <c r="H41" s="44"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="str">
@@ -6981,16 +7017,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B50" s="40" t="str">
+      <c r="B50" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C50" s="41"/>
-      <c r="D50" s="41"/>
-      <c r="E50" s="41"/>
-      <c r="F50" s="41"/>
-      <c r="G50" s="41"/>
-      <c r="H50" s="42"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="43"/>
+      <c r="E50" s="43"/>
+      <c r="F50" s="43"/>
+      <c r="G50" s="43"/>
+      <c r="H50" s="44"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="str">
@@ -7140,16 +7176,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B59" s="40" t="str">
+      <c r="B59" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C59" s="41"/>
-      <c r="D59" s="41"/>
-      <c r="E59" s="41"/>
-      <c r="F59" s="41"/>
-      <c r="G59" s="41"/>
-      <c r="H59" s="42"/>
+      <c r="C59" s="43"/>
+      <c r="D59" s="43"/>
+      <c r="E59" s="43"/>
+      <c r="F59" s="43"/>
+      <c r="G59" s="43"/>
+      <c r="H59" s="44"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="str">
@@ -7295,16 +7331,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B68" s="40" t="str">
+      <c r="B68" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C68" s="41"/>
-      <c r="D68" s="41"/>
-      <c r="E68" s="41"/>
-      <c r="F68" s="41"/>
-      <c r="G68" s="41"/>
-      <c r="H68" s="42"/>
+      <c r="C68" s="43"/>
+      <c r="D68" s="43"/>
+      <c r="E68" s="43"/>
+      <c r="F68" s="43"/>
+      <c r="G68" s="43"/>
+      <c r="H68" s="44"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="str">
@@ -7450,16 +7486,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B77" s="40" t="str">
+      <c r="B77" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C77" s="41"/>
-      <c r="D77" s="41"/>
-      <c r="E77" s="41"/>
-      <c r="F77" s="41"/>
-      <c r="G77" s="41"/>
-      <c r="H77" s="42"/>
+      <c r="C77" s="43"/>
+      <c r="D77" s="43"/>
+      <c r="E77" s="43"/>
+      <c r="F77" s="43"/>
+      <c r="G77" s="43"/>
+      <c r="H77" s="44"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="str">
@@ -7601,16 +7637,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B86" s="40" t="str">
+      <c r="B86" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C86" s="41"/>
-      <c r="D86" s="41"/>
-      <c r="E86" s="41"/>
-      <c r="F86" s="41"/>
-      <c r="G86" s="41"/>
-      <c r="H86" s="42"/>
+      <c r="C86" s="43"/>
+      <c r="D86" s="43"/>
+      <c r="E86" s="43"/>
+      <c r="F86" s="43"/>
+      <c r="G86" s="43"/>
+      <c r="H86" s="44"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="str">
@@ -7749,17 +7785,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B32:H32"/>
     <mergeCell ref="B86:H86"/>
     <mergeCell ref="B41:H41"/>
     <mergeCell ref="B50:H50"/>
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B68:H68"/>
     <mergeCell ref="B77:H77"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B32:H32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -8039,32 +8075,32 @@
         <f>Total!$F$1</f>
         <v>Week 2</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -8222,16 +8258,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -8385,16 +8421,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -8562,16 +8598,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -8723,16 +8759,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -8888,16 +8924,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -9051,16 +9087,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -9210,16 +9246,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="40" t="str">
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -9363,16 +9399,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -9514,16 +9550,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -9662,17 +9698,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9947,32 +9983,32 @@
         <f>Total!$G$1</f>
         <v>Week 3</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -10138,16 +10174,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -10305,16 +10341,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -10472,16 +10508,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -10635,16 +10671,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -10806,16 +10842,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -10973,16 +11009,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -11134,16 +11170,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="40" t="str">
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -11293,16 +11329,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -11444,16 +11480,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -11592,17 +11628,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -11877,32 +11913,32 @@
         <f>Total!$H$1</f>
         <v>Week 4</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -12062,16 +12098,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -12225,16 +12261,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -12390,16 +12426,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -12549,16 +12585,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -12710,16 +12746,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -12873,16 +12909,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -13032,16 +13068,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="40" t="str">
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -13191,16 +13227,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -13342,16 +13378,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -13490,17 +13526,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -13775,31 +13811,31 @@
         <f>Total!$I$1</f>
         <v>Week 5</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -13971,16 +14007,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -14142,16 +14178,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -14323,16 +14359,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -14478,16 +14514,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -14639,16 +14675,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -14802,16 +14838,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -14965,16 +15001,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="40" t="str">
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -15130,16 +15166,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -15281,16 +15317,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -15429,17 +15465,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -15714,32 +15750,32 @@
         <f>Total!$J$1</f>
         <v>Week 6</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -15831,16 +15867,20 @@
       </c>
     </row>
     <row r="8" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="9"/>
+      <c r="A8" s="9" t="s">
+        <v>109</v>
+      </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
+      <c r="G8" s="10">
+        <v>2</v>
+      </c>
       <c r="H8" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -15883,11 +15923,11 @@
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -15905,16 +15945,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -16004,16 +16044,20 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="9"/>
+      <c r="A17" s="9" t="s">
+        <v>105</v>
+      </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10">
+        <v>3</v>
+      </c>
       <c r="H17" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -16056,11 +16100,11 @@
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16068,16 +16112,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -16235,16 +16279,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -16317,16 +16361,20 @@
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="9"/>
+      <c r="A34" s="9" t="s">
+        <v>104</v>
+      </c>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
+      <c r="G34" s="10">
+        <v>3</v>
+      </c>
       <c r="H34" s="6">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -16382,11 +16430,11 @@
       </c>
       <c r="G37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H37" s="11">
         <f>SUM(B37:G37)</f>
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -16394,16 +16442,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -16559,16 +16607,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -16718,16 +16766,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -16877,16 +16925,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="40" t="str">
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -17038,16 +17086,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -17189,16 +17237,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -17337,17 +17385,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -17622,32 +17670,32 @@
         <f>Total!$K$1</f>
         <v>Week 7</v>
       </c>
-      <c r="B1" s="43" t="str">
+      <c r="B1" s="40" t="str">
         <f>'Week (1)'!$B$1</f>
         <v>Total hours</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="str">
         <f>Total!D2</f>
         <v>Nestoras</v>
       </c>
-      <c r="B3" s="40" t="str">
+      <c r="B3" s="42" t="str">
         <f>'Week (1)'!$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="str">
@@ -17684,29 +17732,39 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10">
+        <v>1.5</v>
+      </c>
       <c r="G5" s="10"/>
       <c r="H5" s="6">
         <f>SUM(B5:G5)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
+      <c r="A6" s="9" t="s">
+        <v>108</v>
+      </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="E6" s="10">
+        <v>2</v>
+      </c>
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="6">
         <f t="shared" ref="H6:H9" si="0">SUM(B6:G6)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -17755,7 +17813,7 @@
       </c>
       <c r="B10" s="11">
         <f t="shared" ref="B10:G10" si="1">SUM(B5:B9)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C10" s="11">
         <f t="shared" si="1"/>
@@ -17767,11 +17825,11 @@
       </c>
       <c r="E10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
@@ -17779,7 +17837,7 @@
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -17797,16 +17855,16 @@
         <f>Total!D3</f>
         <v>Denys</v>
       </c>
-      <c r="B12" s="40" t="str">
+      <c r="B12" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="str">
@@ -17843,29 +17901,41 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="F14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G14" s="10"/>
       <c r="H14" s="6">
         <f>SUM(B14:G14)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
+      <c r="A15" s="9" t="s">
+        <v>108</v>
+      </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
+      <c r="E15" s="10">
+        <v>1</v>
+      </c>
+      <c r="F15" s="10">
+        <v>1</v>
+      </c>
       <c r="G15" s="10"/>
       <c r="H15" s="6">
         <f t="shared" ref="H15:H18" si="2">SUM(B15:G15)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
@@ -17914,7 +17984,7 @@
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:G19" si="3">SUM(B14:B18)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="3"/>
@@ -17926,11 +17996,11 @@
       </c>
       <c r="E19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
@@ -17938,7 +18008,7 @@
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -17946,16 +18016,16 @@
         <f>Total!D4</f>
         <v>Jan</v>
       </c>
-      <c r="B21" s="40" t="str">
+      <c r="B21" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
@@ -17992,21 +18062,31 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="F23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G23" s="10"/>
       <c r="H23" s="6">
         <f>SUM(B23:G23)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
+      <c r="A24" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" s="10">
+        <v>1</v>
+      </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
@@ -18014,33 +18094,45 @@
       <c r="G24" s="10"/>
       <c r="H24" s="6">
         <f t="shared" ref="H24:H27" si="4">SUM(B24:G24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="9"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
+      <c r="A25" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="C25" s="10">
+        <v>0.5</v>
+      </c>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="9"/>
+      <c r="A26" s="9" t="s">
+        <v>100</v>
+      </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
+      <c r="E26" s="10">
+        <v>1</v>
+      </c>
+      <c r="F26" s="10">
+        <v>1.5</v>
+      </c>
       <c r="G26" s="10"/>
       <c r="H26" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -18063,11 +18155,11 @@
       </c>
       <c r="B28" s="11">
         <f t="shared" ref="B28:G28" si="5">SUM(B23:B27)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D28" s="11">
         <f t="shared" si="5"/>
@@ -18075,11 +18167,11 @@
       </c>
       <c r="E28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
@@ -18087,7 +18179,7 @@
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18095,16 +18187,16 @@
         <f>Total!D5</f>
         <v>Kirill</v>
       </c>
-      <c r="B30" s="40" t="str">
+      <c r="B30" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="44"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="str">
@@ -18141,29 +18233,39 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="9"/>
+      <c r="A32" s="9" t="s">
+        <v>50</v>
+      </c>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="F32" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G32" s="10"/>
       <c r="H32" s="6">
         <f>SUM(B32:G32)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="9"/>
+      <c r="A33" s="9" t="s">
+        <v>104</v>
+      </c>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
+      <c r="E33" s="10">
+        <v>2</v>
+      </c>
+      <c r="F33" s="10">
+        <v>1</v>
+      </c>
       <c r="G33" s="10"/>
       <c r="H33" s="6">
         <f t="shared" ref="H33:H36" si="6">SUM(B33:G33)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
@@ -18224,11 +18326,11 @@
       </c>
       <c r="E37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="G37" s="11">
         <f t="shared" si="7"/>
@@ -18236,7 +18338,7 @@
       </c>
       <c r="H37" s="11">
         <f>SUM(B37:G37)</f>
-        <v>0</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18244,16 +18346,16 @@
         <f>Total!D6</f>
         <v>Ilya</v>
       </c>
-      <c r="B39" s="40" t="str">
+      <c r="B39" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="42"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="44"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="str">
@@ -18291,37 +18393,48 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B41" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
+      <c r="F41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G41" s="10"/>
       <c r="H41" s="6">
         <f>SUM(B41:G41)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="9"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
+      <c r="A42" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="10">
+        <v>2</v>
+      </c>
+      <c r="C42" s="10">
+        <v>1</v>
+      </c>
       <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
+      <c r="E42" s="10">
+        <v>1</v>
+      </c>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
       <c r="H42" s="6">
         <f t="shared" ref="H42:H45" si="9">SUM(B42:G42)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
@@ -18363,11 +18476,11 @@
       </c>
       <c r="B46" s="11">
         <f t="shared" ref="B46:G46" si="10">SUM(B41:B45)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="C46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" s="11">
         <f t="shared" si="10"/>
@@ -18375,11 +18488,11 @@
       </c>
       <c r="E46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
@@ -18387,7 +18500,7 @@
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18395,16 +18508,16 @@
         <f>Total!D7</f>
         <v>Yevheniia</v>
       </c>
-      <c r="B48" s="40" t="str">
+      <c r="B48" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="44"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="str">
@@ -18442,43 +18555,55 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
+      <c r="F50" s="10">
+        <v>2</v>
+      </c>
       <c r="G50" s="10"/>
       <c r="H50" s="6">
         <f>SUM(B50:G50)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="9"/>
+      <c r="A51" s="9" t="s">
+        <v>106</v>
+      </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
       <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
+      <c r="E51" s="10">
+        <v>2</v>
+      </c>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
       <c r="H51" s="6">
         <f t="shared" ref="H51:H54" si="12">SUM(B51:G51)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" s="9"/>
+      <c r="A52" s="9" t="s">
+        <v>107</v>
+      </c>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
+      <c r="E52" s="10">
+        <v>0.5</v>
+      </c>
       <c r="F52" s="10"/>
       <c r="G52" s="10"/>
       <c r="H52" s="6">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
@@ -18514,7 +18639,7 @@
       </c>
       <c r="B55" s="11">
         <f t="shared" ref="B55:G55" si="13">SUM(B50:B54)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C55" s="11">
         <f t="shared" si="13"/>
@@ -18526,11 +18651,11 @@
       </c>
       <c r="E55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="F55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
@@ -18538,7 +18663,7 @@
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18546,16 +18671,16 @@
         <f>Total!D8</f>
         <v>Fedor</v>
       </c>
-      <c r="B57" s="40" t="str">
+      <c r="B57" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C57" s="41"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="E57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="44"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="str">
@@ -18593,30 +18718,40 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
+      <c r="F59" s="10">
+        <v>2</v>
+      </c>
       <c r="G59" s="10"/>
       <c r="H59" s="6">
         <f>SUM(B59:G59)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
+      <c r="A60" s="9" t="s">
+        <v>103</v>
+      </c>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
       <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
+      <c r="E60" s="10">
+        <v>3</v>
+      </c>
+      <c r="F60" s="10">
+        <v>6</v>
+      </c>
       <c r="G60" s="10"/>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -18665,7 +18800,7 @@
       </c>
       <c r="B64" s="11">
         <f t="shared" ref="B64:G64" si="16">SUM(B59:B63)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C64" s="11">
         <f t="shared" si="16"/>
@@ -18677,11 +18812,11 @@
       </c>
       <c r="E64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
@@ -18689,7 +18824,7 @@
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>0</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18697,16 +18832,16 @@
         <f>Total!D9</f>
         <v>Rokas</v>
       </c>
-      <c r="B66" s="40" t="str">
+      <c r="B66" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C66" s="41"/>
-      <c r="D66" s="41"/>
-      <c r="E66" s="41"/>
-      <c r="F66" s="41"/>
-      <c r="G66" s="41"/>
-      <c r="H66" s="42"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="43"/>
+      <c r="H66" s="44"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="str">
@@ -18744,30 +18879,36 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="B68" s="10"/>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
+      <c r="F68" s="10">
+        <v>1.5</v>
+      </c>
       <c r="G68" s="10"/>
       <c r="H68" s="6">
         <f>SUM(B68:G68)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="9"/>
+      <c r="A69" s="9" t="s">
+        <v>101</v>
+      </c>
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
+      <c r="D69" s="10">
+        <v>2</v>
+      </c>
       <c r="E69" s="10"/>
       <c r="F69" s="10"/>
       <c r="G69" s="10"/>
       <c r="H69" s="6">
         <f t="shared" ref="H69:H72" si="18">SUM(B69:G69)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -18824,7 +18965,7 @@
       </c>
       <c r="D73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E73" s="11">
         <f t="shared" si="19"/>
@@ -18832,7 +18973,7 @@
       </c>
       <c r="F73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
@@ -18840,7 +18981,7 @@
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18848,16 +18989,16 @@
         <f>Total!D10</f>
         <v>0</v>
       </c>
-      <c r="B75" s="40" t="str">
+      <c r="B75" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C75" s="41"/>
-      <c r="D75" s="41"/>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="41"/>
-      <c r="H75" s="42"/>
+      <c r="C75" s="43"/>
+      <c r="D75" s="43"/>
+      <c r="E75" s="43"/>
+      <c r="F75" s="43"/>
+      <c r="G75" s="43"/>
+      <c r="H75" s="44"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="str">
@@ -18999,16 +19140,16 @@
         <f>Total!D11</f>
         <v>0</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="42" t="str">
         <f>$B$3</f>
         <v>Hours</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="41"/>
-      <c r="F84" s="41"/>
-      <c r="G84" s="41"/>
-      <c r="H84" s="42"/>
+      <c r="C84" s="43"/>
+      <c r="D84" s="43"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="44"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="str">
@@ -19147,17 +19288,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B30:H30"/>
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B75:H75"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -19165,26 +19306,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <c6664f9864b54a78bdf9e6230de1c78b xmlns="6c73e52c-07d4-4617-ab67-464747257e8d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </c6664f9864b54a78bdf9e6230de1c78b>
-    <Versiebeheer xmlns="ab37b2fe-4f81-426e-b942-40459dbac68c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100294690D6A57C3C4B8650464765815F1C" ma:contentTypeVersion="15" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="bf1d2ff51e740e451b46e7c13bf9e6da">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="45f6ce90-ba85-4ef2-b43f-c64448cd95eb" xmlns:ns3="c7549584-aa9c-449c-abfe-2ca02f3a7188" xmlns:ns4="6c73e52c-07d4-4617-ab67-464747257e8d" xmlns:ns5="ab37b2fe-4f81-426e-b942-40459dbac68c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8575fd65d7959dd12bd4dc11d36e634e" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="45f6ce90-ba85-4ef2-b43f-c64448cd95eb"/>
@@ -19427,26 +19548,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{844B94A5-2CB8-4D3A-A97F-85854BBCA257}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <c6664f9864b54a78bdf9e6230de1c78b xmlns="6c73e52c-07d4-4617-ab67-464747257e8d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </c6664f9864b54a78bdf9e6230de1c78b>
+    <Versiebeheer xmlns="ab37b2fe-4f81-426e-b942-40459dbac68c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477D1558-F7E0-401F-8472-E1151A96BE17}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c73e52c-07d4-4617-ab67-464747257e8d"/>
-    <ds:schemaRef ds:uri="ab37b2fe-4f81-426e-b942-40459dbac68c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{724CCB8E-5E6A-4B8C-A558-5D9223ADF390}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19465,4 +19587,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477D1558-F7E0-401F-8472-E1151A96BE17}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c73e52c-07d4-4617-ab67-464747257e8d"/>
+    <ds:schemaRef ds:uri="ab37b2fe-4f81-426e-b942-40459dbac68c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{844B94A5-2CB8-4D3A-A97F-85854BBCA257}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the hour log for the week 8.
</commit_message>
<xml_diff>
--- a/docs/2.2_P.CoB_Time_registration_for10.xlsx
+++ b/docs/2.2_P.CoB_Time_registration_for10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shawn\Dev\ClientOnBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6518D0F2-3554-44C2-BA4D-D03CC9C562E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD32A7F6-5AFB-4967-9912-247212F64384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="835" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructie" sheetId="19" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="134">
   <si>
     <t>Kickoff</t>
   </si>
@@ -373,6 +373,78 @@
   </si>
   <si>
     <t>Rendering the list of history entries in the action bar</t>
+  </si>
+  <si>
+    <t>Reviewing work of teammates, providing help</t>
+  </si>
+  <si>
+    <t>Refining requirements in functional design</t>
+  </si>
+  <si>
+    <t>Creating frontend for inviting members</t>
+  </si>
+  <si>
+    <t>Creating frontend for inviting users</t>
+  </si>
+  <si>
+    <t>Creating backedn and frontend for removing users from a session</t>
+  </si>
+  <si>
+    <t>Frontend for changing emails</t>
+  </si>
+  <si>
+    <t>Fixing Postman setup</t>
+  </si>
+  <si>
+    <t>Tests for backend for deleting other users</t>
+  </si>
+  <si>
+    <t>Socket notification for a closed session</t>
+  </si>
+  <si>
+    <t>Functionality to support disabled editor for closed session</t>
+  </si>
+  <si>
+    <t>Real-time synchronization of the editor state</t>
+  </si>
+  <si>
+    <t>Helping Nestoras with his task</t>
+  </si>
+  <si>
+    <t>Helping Denys with his task</t>
+  </si>
+  <si>
+    <t>Frontend of statistics page</t>
+  </si>
+  <si>
+    <t>Fixing issues with the application, adding missing functionality</t>
+  </si>
+  <si>
+    <t>Team outcome, refining team plan, writing missing documentation</t>
+  </si>
+  <si>
+    <t>Documenting security architecture</t>
+  </si>
+  <si>
+    <t>Addressing client's feedback on wireframes</t>
+  </si>
+  <si>
+    <t>Page for changing password</t>
+  </si>
+  <si>
+    <t>Reviewing work of teammates</t>
+  </si>
+  <si>
+    <t>Documenting libraries</t>
+  </si>
+  <si>
+    <t>Writing deployment manual</t>
+  </si>
+  <si>
+    <t>Frontend for deleting other users</t>
+  </si>
+  <si>
+    <t>Writing acceptance tests and executing them</t>
   </si>
 </sst>
 </file>
@@ -992,10 +1064,10 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1081,7 +1153,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>9.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1164,10 +1236,10 @@
                   <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>9.5</c:v>
+                  <c:v>10.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1253,7 +1325,7 @@
                   <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1336,10 +1408,10 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>9</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1422,10 +1494,10 @@
                   <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1508,10 +1580,10 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13.5</c:v>
+                  <c:v>21.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>25.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1594,10 +1666,10 @@
                   <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.5</c:v>
+                  <c:v>8.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2005,10 +2077,10 @@
                   <c:v>345.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>284.5</c:v>
+                  <c:v>262.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>284.5</c:v>
+                  <c:v>144</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3609,55 +3681,75 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G5" s="10"/>
       <c r="H5" s="6">
         <f>SUM(B5:G5)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
+      <c r="A6" s="9" t="s">
+        <v>123</v>
+      </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
+      <c r="E6" s="10">
+        <v>8</v>
+      </c>
+      <c r="F6" s="10">
+        <v>1</v>
+      </c>
       <c r="G6" s="10"/>
       <c r="H6" s="6">
         <f t="shared" ref="H6:H9" si="0">SUM(B6:G6)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="9"/>
+      <c r="A7" s="9" t="s">
+        <v>129</v>
+      </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+      <c r="G7" s="10">
+        <v>0.5</v>
+      </c>
       <c r="H7" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="9"/>
+      <c r="A8" s="9" t="s">
+        <v>130</v>
+      </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
+      <c r="G8" s="10">
+        <v>0.5</v>
+      </c>
       <c r="H8" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -3680,7 +3772,7 @@
       </c>
       <c r="B10" s="11">
         <f t="shared" ref="B10:G10" si="1">SUM(B5:B9)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C10" s="11">
         <f t="shared" si="1"/>
@@ -3692,19 +3784,19 @@
       </c>
       <c r="E10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -3768,55 +3860,75 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="F14" s="10">
+        <v>2</v>
+      </c>
       <c r="G14" s="10"/>
       <c r="H14" s="6">
         <f>SUM(B14:G14)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="10">
+        <v>1</v>
+      </c>
       <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="D15" s="10">
+        <v>2</v>
+      </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="6">
         <f t="shared" ref="H15:H18" si="2">SUM(B15:G15)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
+      <c r="A16" s="9" t="s">
+        <v>127</v>
+      </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
+      <c r="F16" s="10">
+        <v>1</v>
+      </c>
       <c r="G16" s="10"/>
       <c r="H16" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="9"/>
+      <c r="A17" s="9" t="s">
+        <v>128</v>
+      </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10">
+        <v>1</v>
+      </c>
       <c r="H17" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -3839,7 +3951,7 @@
       </c>
       <c r="B19" s="11">
         <f t="shared" ref="B19:G19" si="3">SUM(B14:B18)</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="3"/>
@@ -3847,7 +3959,7 @@
       </c>
       <c r="D19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E19" s="11">
         <f t="shared" si="3"/>
@@ -3855,15 +3967,15 @@
       </c>
       <c r="F19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="11">
         <f>SUM(B19:G19)</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -3917,68 +4029,100 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="F23" s="10">
+        <v>2.5</v>
+      </c>
       <c r="G23" s="10"/>
       <c r="H23" s="6">
         <f>SUM(B23:G23)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
+      <c r="A24" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" s="10">
+        <v>0.5</v>
+      </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
+      <c r="E24" s="10">
+        <v>2</v>
+      </c>
+      <c r="F24" s="10">
+        <v>2</v>
+      </c>
       <c r="G24" s="10"/>
       <c r="H24" s="6">
         <f t="shared" ref="H24:H27" si="4">SUM(B24:G24)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="9"/>
+      <c r="A25" s="9" t="s">
+        <v>110</v>
+      </c>
       <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
+      <c r="C25" s="10">
+        <v>0.5</v>
+      </c>
       <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
+      <c r="E25" s="10">
+        <v>1</v>
+      </c>
+      <c r="F25" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="G25" s="10">
+        <v>1.5</v>
+      </c>
       <c r="H25" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="9"/>
+      <c r="A26" s="9" t="s">
+        <v>124</v>
+      </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
+      <c r="G26" s="10">
+        <v>2.5</v>
+      </c>
       <c r="H26" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="9"/>
+      <c r="A27" s="9" t="s">
+        <v>125</v>
+      </c>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10">
+        <v>2.5</v>
+      </c>
       <c r="H27" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="22" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -3988,11 +4132,11 @@
       </c>
       <c r="B28" s="11">
         <f t="shared" ref="B28:G28" si="5">SUM(B23:B27)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D28" s="11">
         <f t="shared" si="5"/>
@@ -4000,19 +4144,19 @@
       </c>
       <c r="E28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -4066,59 +4210,79 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
+      <c r="A32" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="10">
+        <v>2</v>
+      </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="F32" s="10">
+        <v>2</v>
+      </c>
       <c r="G32" s="10"/>
       <c r="H32" s="6">
         <f>SUM(B32:G32)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="9"/>
+      <c r="A33" s="9" t="s">
+        <v>120</v>
+      </c>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
+      <c r="D33" s="10">
+        <v>2</v>
+      </c>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
       <c r="H33" s="6">
         <f t="shared" ref="H33:H36" si="6">SUM(B33:G33)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="9"/>
+      <c r="A34" s="9" t="s">
+        <v>122</v>
+      </c>
       <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
+      <c r="C34" s="10">
+        <v>2</v>
+      </c>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
       <c r="H34" s="6">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="9"/>
+      <c r="A35" s="9" t="s">
+        <v>121</v>
+      </c>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
+      <c r="E35" s="10">
+        <v>1</v>
+      </c>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
       <c r="H35" s="6">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="9"/>
+      <c r="A36" s="9" t="s">
+        <v>103</v>
+      </c>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
@@ -4137,23 +4301,23 @@
       </c>
       <c r="B37" s="11">
         <f t="shared" ref="B37:G37" si="7">SUM(B32:B36)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G37" s="11">
         <f t="shared" si="7"/>
@@ -4161,7 +4325,7 @@
       </c>
       <c r="H37" s="11">
         <f>SUM(B37:G37)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -4216,22 +4380,30 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B41" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B41" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
+      <c r="F41" s="10">
+        <v>2</v>
+      </c>
       <c r="G41" s="10"/>
       <c r="H41" s="6">
         <f>SUM(B41:G41)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="9"/>
-      <c r="B42" s="10"/>
+      <c r="A42" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B42" s="10">
+        <v>2</v>
+      </c>
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
       <c r="E42" s="10"/>
@@ -4239,20 +4411,26 @@
       <c r="G42" s="10"/>
       <c r="H42" s="6">
         <f t="shared" ref="H42:H45" si="9">SUM(B42:G42)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="9"/>
+      <c r="A43" s="9" t="s">
+        <v>114</v>
+      </c>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
+      <c r="D43" s="10">
+        <v>1</v>
+      </c>
+      <c r="E43" s="10">
+        <v>6.5</v>
+      </c>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
       <c r="H43" s="6">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -4288,7 +4466,7 @@
       </c>
       <c r="B46" s="11">
         <f t="shared" ref="B46:G46" si="10">SUM(B41:B45)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="C46" s="11">
         <f t="shared" si="10"/>
@@ -4296,15 +4474,15 @@
       </c>
       <c r="D46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="F46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
@@ -4312,7 +4490,7 @@
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -4367,43 +4545,55 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B50" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C50" s="10"/>
       <c r="D50" s="10"/>
       <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
+      <c r="F50" s="10">
+        <v>2</v>
+      </c>
       <c r="G50" s="10"/>
       <c r="H50" s="6">
         <f>SUM(B50:G50)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="9"/>
+      <c r="A51" s="9" t="s">
+        <v>119</v>
+      </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
+      <c r="D51" s="10">
+        <v>2</v>
+      </c>
       <c r="E51" s="10"/>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
       <c r="H51" s="6">
         <f t="shared" ref="H51:H54" si="12">SUM(B51:G51)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" s="9"/>
+      <c r="A52" s="9" t="s">
+        <v>126</v>
+      </c>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="10"/>
       <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
+      <c r="F52" s="10">
+        <v>1</v>
+      </c>
       <c r="G52" s="10"/>
       <c r="H52" s="6">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
@@ -4439,7 +4629,7 @@
       </c>
       <c r="B55" s="11">
         <f t="shared" ref="B55:G55" si="13">SUM(B50:B54)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C55" s="11">
         <f t="shared" si="13"/>
@@ -4447,7 +4637,7 @@
       </c>
       <c r="D55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E55" s="11">
         <f t="shared" si="13"/>
@@ -4455,7 +4645,7 @@
       </c>
       <c r="F55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
@@ -4463,7 +4653,7 @@
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -4518,56 +4708,78 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B59" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
+      <c r="F59" s="10">
+        <v>2</v>
+      </c>
       <c r="G59" s="10"/>
       <c r="H59" s="6">
         <f>SUM(B59:G59)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="9"/>
+      <c r="A60" s="9" t="s">
+        <v>103</v>
+      </c>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
+      <c r="D60" s="10">
+        <v>6</v>
+      </c>
+      <c r="E60" s="10">
+        <v>2</v>
+      </c>
+      <c r="F60" s="10">
+        <v>3</v>
+      </c>
+      <c r="G60" s="10">
+        <v>8</v>
+      </c>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A61" s="9"/>
+      <c r="A61" s="9" t="s">
+        <v>131</v>
+      </c>
       <c r="B61" s="10"/>
       <c r="C61" s="10"/>
       <c r="D61" s="10"/>
       <c r="E61" s="10"/>
       <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
+      <c r="G61" s="10">
+        <v>1</v>
+      </c>
       <c r="H61" s="6">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A62" s="9"/>
+      <c r="A62" s="9" t="s">
+        <v>129</v>
+      </c>
       <c r="B62" s="10"/>
       <c r="C62" s="10"/>
       <c r="D62" s="10"/>
       <c r="E62" s="10"/>
       <c r="F62" s="10"/>
-      <c r="G62" s="10"/>
+      <c r="G62" s="10">
+        <v>1</v>
+      </c>
       <c r="H62" s="6">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
@@ -4590,7 +4802,7 @@
       </c>
       <c r="B64" s="11">
         <f t="shared" ref="B64:G64" si="16">SUM(B59:B63)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C64" s="11">
         <f t="shared" si="16"/>
@@ -4598,23 +4810,23 @@
       </c>
       <c r="D64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>0</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -4669,56 +4881,74 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="10"/>
+        <v>50</v>
+      </c>
+      <c r="B68" s="10">
+        <v>2.5</v>
+      </c>
       <c r="C68" s="10"/>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
+      <c r="F68" s="10">
+        <v>2</v>
+      </c>
       <c r="G68" s="10"/>
       <c r="H68" s="6">
         <f>SUM(B68:G68)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="9"/>
+      <c r="A69" s="9" t="s">
+        <v>117</v>
+      </c>
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
+      <c r="D69" s="10">
+        <v>1</v>
+      </c>
       <c r="E69" s="10"/>
-      <c r="F69" s="10"/>
+      <c r="F69" s="10">
+        <v>1.5</v>
+      </c>
       <c r="G69" s="10"/>
       <c r="H69" s="6">
         <f t="shared" ref="H69:H72" si="18">SUM(B69:G69)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" s="9"/>
+      <c r="A70" s="9" t="s">
+        <v>132</v>
+      </c>
       <c r="B70" s="10"/>
       <c r="C70" s="10"/>
       <c r="D70" s="10"/>
       <c r="E70" s="10"/>
-      <c r="F70" s="10"/>
+      <c r="F70" s="10">
+        <v>1.5</v>
+      </c>
       <c r="G70" s="10"/>
       <c r="H70" s="6">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" s="9"/>
+      <c r="A71" s="9" t="s">
+        <v>133</v>
+      </c>
       <c r="B71" s="10"/>
       <c r="C71" s="10"/>
       <c r="D71" s="10"/>
       <c r="E71" s="10"/>
       <c r="F71" s="10"/>
-      <c r="G71" s="10"/>
+      <c r="G71" s="10">
+        <v>10</v>
+      </c>
       <c r="H71" s="6">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
@@ -4727,11 +4957,13 @@
       <c r="C72" s="10"/>
       <c r="D72" s="10"/>
       <c r="E72" s="10"/>
-      <c r="F72" s="10"/>
+      <c r="F72" s="10">
+        <v>1.5</v>
+      </c>
       <c r="G72" s="10"/>
       <c r="H72" s="6">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
@@ -4741,7 +4973,7 @@
       </c>
       <c r="B73" s="11">
         <f t="shared" ref="B73:G73" si="19">SUM(B68:B72)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="C73" s="11">
         <f t="shared" si="19"/>
@@ -4749,7 +4981,7 @@
       </c>
       <c r="D73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E73" s="11">
         <f t="shared" si="19"/>
@@ -4757,15 +4989,15 @@
       </c>
       <c r="F73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -5362,15 +5594,15 @@
       </c>
       <c r="K2" s="3">
         <f>'Week (7)'!$H$10</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L2" s="3">
         <f>'Week (8)'!$H$10</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="M2" s="4">
         <f>SUM(E2:L2)</f>
-        <v>53.5</v>
+        <v>72.5</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5409,11 +5641,11 @@
       </c>
       <c r="L3" s="3">
         <f>'Week (8)'!$H$19</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="M3" s="4">
         <f t="shared" ref="M3:M5" si="0">SUM(E3:L3)</f>
-        <v>58.5</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5452,15 +5684,15 @@
       </c>
       <c r="K4" s="3">
         <f>'Week (7)'!$H$28</f>
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="L4" s="3">
         <f>'Week (8)'!$H$28</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>78</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -5499,11 +5731,11 @@
       </c>
       <c r="L5" s="3">
         <f>'Week (8)'!$H$37</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>48.5</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5538,15 +5770,15 @@
       </c>
       <c r="K6" s="3">
         <f>'Week (7)'!$H$46</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L6" s="3">
         <f>'Week (8)'!$H$46</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="M6" s="4">
         <f t="shared" ref="M6" si="1">SUM(E6:L6)</f>
-        <v>69</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5581,15 +5813,15 @@
       </c>
       <c r="K7" s="3">
         <f>'Week (7)'!$H$55</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L7" s="3">
         <f>'Week (8)'!$H$55</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="M7" s="4">
         <f t="shared" ref="M7:M11" si="2">SUM(E7:L7)</f>
-        <v>66</v>
+        <v>74.5</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5624,15 +5856,15 @@
       </c>
       <c r="K8" s="3">
         <f>'Week (7)'!$H$64</f>
-        <v>13.5</v>
+        <v>21.5</v>
       </c>
       <c r="L8" s="3">
         <f>'Week (8)'!$H$64</f>
-        <v>0</v>
+        <v>25.5</v>
       </c>
       <c r="M8" s="4">
         <f t="shared" si="2"/>
-        <v>64.5</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5667,15 +5899,15 @@
       </c>
       <c r="K9" s="3">
         <f>'Week (7)'!$H$73</f>
-        <v>3.5</v>
+        <v>8.5</v>
       </c>
       <c r="L9" s="3">
         <f>'Week (8)'!$H$73</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M9" s="4">
         <f t="shared" si="2"/>
-        <v>45.5</v>
+        <v>70.5</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5792,11 +6024,11 @@
       </c>
       <c r="K12" s="15">
         <f t="shared" si="3"/>
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="L12" s="15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>118.5</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5823,7 +6055,7 @@
       <c r="K13" s="20"/>
       <c r="L13" s="20">
         <f>SUM(K12:L12)</f>
-        <v>61</v>
+        <v>201.5</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5858,11 +6090,11 @@
       </c>
       <c r="K14" s="18">
         <f t="shared" si="4"/>
-        <v>284.5</v>
+        <v>262.5</v>
       </c>
       <c r="L14" s="18">
         <f t="shared" si="4"/>
-        <v>284.5</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -17761,10 +17993,12 @@
         <v>2</v>
       </c>
       <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
+      <c r="G6" s="10">
+        <v>4</v>
+      </c>
       <c r="H6" s="6">
         <f t="shared" ref="H6:H9" si="0">SUM(B6:G6)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -17833,11 +18067,11 @@
       </c>
       <c r="G10" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H10" s="11">
         <f>SUM(B10:G10)</f>
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -18136,16 +18370,20 @@
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="9"/>
+      <c r="A27" s="9" t="s">
+        <v>110</v>
+      </c>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10">
+        <v>1</v>
+      </c>
       <c r="H27" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="22" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -18175,11 +18413,11 @@
       </c>
       <c r="G28" s="11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" s="11">
         <f>SUM(B28:G28)</f>
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18432,15 +18670,19 @@
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="9"/>
+      <c r="A43" s="9" t="s">
+        <v>112</v>
+      </c>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
+      <c r="G43" s="10">
+        <v>3</v>
+      </c>
       <c r="H43" s="6">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -18496,11 +18738,11 @@
       </c>
       <c r="G46" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H46" s="11">
         <f>SUM(B46:G46)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18607,16 +18849,20 @@
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" s="9"/>
+      <c r="A53" s="9" t="s">
+        <v>118</v>
+      </c>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
       <c r="D53" s="10"/>
       <c r="E53" s="10"/>
       <c r="F53" s="10"/>
-      <c r="G53" s="10"/>
+      <c r="G53" s="10">
+        <v>1</v>
+      </c>
       <c r="H53" s="6">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
@@ -18659,11 +18905,11 @@
       </c>
       <c r="G55" s="11">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H55" s="11">
         <f>SUM(B55:G55)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18748,10 +18994,12 @@
       <c r="F60" s="10">
         <v>6</v>
       </c>
-      <c r="G60" s="10"/>
+      <c r="G60" s="10">
+        <v>8</v>
+      </c>
       <c r="H60" s="6">
         <f t="shared" ref="H60:H63" si="15">SUM(B60:G60)</f>
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -18820,11 +19068,11 @@
       </c>
       <c r="G64" s="11">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H64" s="11">
         <f>SUM(B64:G64)</f>
-        <v>13.5</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">
@@ -18912,29 +19160,37 @@
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" s="9"/>
+      <c r="A70" s="9" t="s">
+        <v>115</v>
+      </c>
       <c r="B70" s="10"/>
       <c r="C70" s="10"/>
       <c r="D70" s="10"/>
       <c r="E70" s="10"/>
       <c r="F70" s="10"/>
-      <c r="G70" s="10"/>
+      <c r="G70" s="10">
+        <v>2</v>
+      </c>
       <c r="H70" s="6">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" s="9"/>
+      <c r="A71" s="9" t="s">
+        <v>116</v>
+      </c>
       <c r="B71" s="10"/>
       <c r="C71" s="10"/>
       <c r="D71" s="10"/>
       <c r="E71" s="10"/>
       <c r="F71" s="10"/>
-      <c r="G71" s="10"/>
+      <c r="G71" s="10">
+        <v>3</v>
+      </c>
       <c r="H71" s="6">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
@@ -18977,11 +19233,11 @@
       </c>
       <c r="G73" s="11">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H73" s="11">
         <f>SUM(B73:G73)</f>
-        <v>3.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.2">

</xml_diff>